<commit_message>
In maatregel M01 "Het project levert in elke fase vastgestelde producten en informatie op" verduidelijkt dat de aparte detailtestplannen die onder verantwoordelijkheid van het project door een derde partij worden uitgevoerd doorgaans de vorm hebben van een offerteaanvraag gemaakt door ICTU en een offerte met plan van aanpak gemaakt door de leverancier.
Closes #953.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -157,7 +157,7 @@
 - Template infrastructuurarchitectuur.
 Testplannen en -rapportages
 De testplannen bestaan uit een mastertestplan (MTP), gemaakt op basis van een productrisicoanalyse (PRA), en detailtestplannen. Het doel van een mastertestplan is om betrokkenen bij het testproces te informeren over de strategie, aanpak, activiteiten, inclusief de onderlinge relaties en afhankelijkheden, en de op te leveren producten met betrekking tot het testtraject. Het mastertestplan beschrijft deze strategie, aanpak, activiteiten en eindproducten, die in de detailtestplannen verder worden gedetailleerd.
-De opdrachtgevende organisatie is verantwoordelijk voor het mastertestplan. Het project maakt een detailtestplan voor de testsoorten die tijdens de realisatiefase door het project worden uitgevoerd. Voor testen die onder verantwoordelijkheid van het project door een derde partij worden uitgevoerd, denk aan penetratietesten en evaluaties van gebruikskwaliteit, worden aparte detailtestplannen gemaakt.
+De opdrachtgevende organisatie is verantwoordelijk voor het mastertestplan. Het project maakt een detailtestplan voor de testsoorten die tijdens de realisatiefase door het project worden uitgevoerd. Voor testen die onder verantwoordelijkheid van het project door een derde partij worden uitgevoerd, denk aan penetratietesten en evaluaties van gebruikskwaliteit, worden aparte detailtestplannen gemaakt. Deze hebben doorgaans de vorm van een offerteaanvraag gemaakt door ICTU en een offerte met plan van aanpak gemaakt door de leverancier.
 Logische testgevallen worden vastgelegd en gekoppeld met use cases en user stories. Fysieke testgevallen worden vastgelegd in het formaat van de gebruikte tooling en gekoppeld met de logische testgevallen. Op basis hiervan worden testrapportages gegenereerd die laten zien dat alle use cases en user stories zijn getest en dat die tests zijn geslaagd.
 Beschikbare templates:
 - Template detailtestplan softwarerealisatie.
@@ -884,7 +884,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
   <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 02-08-2024.</t>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 22-10-2024.</t>
   </si>
   <si>
     <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Bij maatregelen met submaatregelen hoeft alleen de status van de submaatregelen te worden ingevuld.</t>

</xml_diff>

<commit_message>
"OWASP ZAP" hernoemd naar "ZAP by Checkmarx" in alle documenten.
Closes #945.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -438,7 +438,7 @@
 8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),
 9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,
 10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,
-11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: OWASP ZAP (Zed Attack Proxy),
+11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,
 12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,
 13. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,
 14. testen op toegankelijkheid van de applicatie: Axe,
@@ -884,7 +884,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
   <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 02-08-2024.</t>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 22-10-2024.</t>
   </si>
   <si>
     <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Bij maatregelen met submaatregelen hoeft alleen de status van de submaatregelen te worden ingevuld.</t>
@@ -1121,7 +1121,7 @@
     <t>10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,</t>
   </si>
   <si>
-    <t>11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: OWASP ZAP (Zed Attack Proxy),</t>
+    <t>11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,</t>
   </si>
   <si>
     <t>12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,</t>

</xml_diff>

<commit_message>
Voeg template voor voortgang voorfase producten toe. (#986)
Closes #760.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -30,10 +30,10 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">M31: Het project beschikt over actuele vastgestelde informatie
-Voor een goede uitvoering van het project is specifieke informatie nodig. De opdrachtgevende organisatie zorgt dat het project bij de start van de voorfase inzicht heeft in de informatie die typisch wordt vastgelegd in een projectstartarchitectuur, business impact analysis en privacy impact assessment. Waar nodig werkt de opdrachtgevende organisatie de informatie bij tijdens de voorfase en realisatiefase.
+Voor een goede uitvoering van het project is specifieke informatie nodig. De opdrachtgevende organisatie zorgt dat het project bij de start van de voorfase inzicht heeft in de informatie die typisch wordt vastgelegd in een projectstartarchitectuur, business impact analyse en privacy impact assessment. Waar nodig werkt de opdrachtgevende organisatie de informatie bij tijdens de voorfase en realisatiefase.
 De opdrachtgevende organisatie zorgt dat het project vanaf de start van de voorfase beschikt over:
 1. Projectstartarchitectuur,
-2. Business impact analysis,
+2. Business impact analyse,
 3. Privacy impact assessment,
 4. Afspraken tussen opdrachtgevende organisatie en beheerorganisatie.
 Als de benodigde informatie niet gereed is bij de start van de voorfase dan maken opdrachtgevende organisatie en ICTU nadere afspraken over de manier waarop de benodigde informatie nog tijdens de voorfase beschikbaar komt voor het project.
@@ -49,8 +49,8 @@
 Zie https://www.noraonline.nl/wiki/PSA.
 Conform NORA werkt de opdrachtgevende organisatie na de start van het project de PSA uit in een solution architectuur (SA).
 Zie https://www.noraonline.nl/wiki/Solution-architectuur.
-Business impact analysis
-In een business impact analysis (BIA) legt de opdrachtgevende organisatie vast hoe belangrijk informatiebeveiliging is voor de eigen bedrijfsvoering/processen. Naast de gevoeligheid voor incidenten komt hierin ook de 'risk appetite' van de organisatie tot uiting: de risico’s die een organisatie bereid is te accepteren. Alleen de opdrachtgevende organisatie zelf kan hierover een uitspraak doen.
+Business impact analyse
+In een business impact analyse (BIA) legt de opdrachtgevende organisatie vast hoe belangrijk informatiebeveiliging is voor de eigen bedrijfsvoering/processen. Naast de gevoeligheid voor incidenten komt hierin ook de 'risk appetite' van de organisatie tot uiting: de risico’s die een organisatie bereid is te accepteren. Alleen de opdrachtgevende organisatie zelf kan hierover een uitspraak doen.
 Privacy impact assessment
 In een privacy impact assessment (PIA) legt de opdrachtgevende organisatie vast wat de privacy-gevoeligheid is van de gegevens die in een proces of informatiesysteem worden verzameld en verwerkt. De rechtmatigheid van de verwerking wordt beoordeeld. En de PIA stelt grenzen aan de gegevens die mogen worden verzameld en verwerkt. Zicht op privacygevoelige gegevens en het (laten) treffen van adequate en afdoende beschermingsmaatregelen is een wettelijke plicht die een organisatie niet aan een andere partij kan overdragen.
 Als een PIA niet nodig is, dan is een verklaring daaromtrent vereist.
@@ -94,7 +94,7 @@
 De onderstaande tabel bevat de in deze paragraaf beschreven producten. Het ✔ geeft aan in welke fase ze worden opgeleverd.
 Product                                             Voor start Voorfase Realisatiefase Verantwoordelijke organisatie 
 Projectstartarchitectuur                            x                                  opdrachtgever                 
-Business impact analysis                            x                                  opdrachtgever                 
+Business impact analyse                             x                                  opdrachtgever                 
 Privacy impact assessment                           x                                  opdrachtgever                 
 Plan van aanpak: voorfase                           x                                  ICTU                          
 Beschrijving van functionele eisen                             x        x              opdrachtgever                 
@@ -112,8 +112,8 @@
 Software bill of materials                                              x              ICTU                          
 Release notes                                                           x              ICTU                          
 Vrijgaveadvies                                                          x              opdrachtgever                 
-Projectstartarchitectuur, business impact analysis en privacy impact assessment
-De opdrachtgevende organisatie zorgt dat het project bij de start van de voorfase inzicht heeft in de informatie die typisch wordt vastgelegd in een projectstartarchitectuur, business impact analysis en privacy impact assessment. Zie M31: Het project beschikt over actuele vastgestelde informatie.
+Projectstartarchitectuur, business impact analyse en privacy impact assessment
+De opdrachtgevende organisatie zorgt dat het project bij de start van de voorfase inzicht heeft in de informatie die typisch wordt vastgelegd in een projectstartarchitectuur, business impact analyse en privacy impact assessment. Zie M31: Het project beschikt over actuele vastgestelde informatie.
 Plan van aanpak
 Het plan van aanpak voor de voorfase en het plan van aanpak voor de realisatiefase beschrijven de in deze fasen te realiseren producten en diensten, en de planning, werkwijze en verantwoordelijkheden voor de totstandkoming van die producten en diensten.
 Als tijdens de realisatiefase van het project bestaande software dient te worden afgebouwd, onderhouden en/of herbouwd, bevat het plan van aanpak voor de voorfase een onderzoek naar de kwaliteit van deze software, zie M32: Het project onderzoekt de kwaliteit van over te nemen software.
@@ -163,7 +163,7 @@
 - Template mastertestplan.
 - Template detailtestplan softwarerealisatie.
 Informatiebeveiligingsplan
-Het informatiebeveiligingsplan vormt een praktisch toepasbaar document dat uitlegt binnen welke kaders bescherming geleverd wordt tegen welke dreigingen en met welke maatregelen die bescherming vorm krijgt. Mogelijke bronnen voor het informatiebeveiligingsplan zijn de business impact analysis (BIA), privacy impact assessment (PIA) en de threat and vulnerability assessment (TVA).
+Het informatiebeveiligingsplan vormt een praktisch toepasbaar document dat uitlegt binnen welke kaders bescherming geleverd wordt tegen welke dreigingen en met welke maatregelen die bescherming vorm krijgt. Mogelijke bronnen voor het informatiebeveiligingsplan zijn de business impact analyse (BIA), privacy impact assessment (PIA) en de threat and vulnerability assessment (TVA).
 Het Besluit Voorschrift Informatiebeveiliging Rijksdienst 2007 (VIR 2007) bevat een methode om te komen tot een systematische aanpak van informatiebeveiliging. Eén van de vereisten van het VIR 2007 is dat voor elk informatiesysteem en voor elk verantwoordelijkheidsgebied een afhankelijkheids- en kwetsbaarheidsanalyse (A&amp;K-analyse) wordt uitgevoerd.
 Bij ICTU wordt daarvoor een TVA gebruikt. Hierin worden de betrouwbaarheidseisen, die aan de bedrijfsprocessen en dientengevolge aan het informatiesysteem of verantwoordelijkheidsgebied worden gesteld, tijdens een afhankelijkheidsanalyse geïnventariseerd. Vervolgens worden de bedreigingen geïdentificeerd en geanalyseerd. De TVA levert zodoende een deel van een traceerbare onderbouwing voor de te treffen beveiligingsmaatregelen. De TVA wordt tijdens de voorfase opgesteld op basis van de resultaten van de BIA, de eventuele PIA en de inhoud van de ontwerp- en architectuurdocumentatie.
 Kwaliteitsplan
@@ -921,7 +921,7 @@
     <t>1. Projectstartarchitectuur,</t>
   </si>
   <si>
-    <t>2. Business impact analysis,</t>
+    <t>2. Business impact analyse,</t>
   </si>
   <si>
     <t>3. Privacy impact assessment,</t>
@@ -939,7 +939,7 @@
     <t>1. Projectstartarchitectuur</t>
   </si>
   <si>
-    <t>2. Business impact analysis</t>
+    <t>2. Business impact analyse</t>
   </si>
   <si>
     <t>3. Privacy impact assessment</t>
@@ -1404,7 +1404,7 @@
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>

</xml_diff>

<commit_message>
Actueel houden externe software.
In maatregel M16 "Het project gebruikt tools voor vastgestelde taken" de taak "actueel houden van externe software" toegevoegd.

Closes #392.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -417,7 +417,7 @@
 5. release van software,
 6. maken van testrapportages,
 7. maken van kwaliteitsrapportages,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden,
+8. actueel houden van externe software,
 9. controleren van door de applicatie gebruikte versies van externe software op aanwezigheid van bekende kwetsbaarheden,
 10. statische controle van de software op aanwezigheid van kwetsbare constructies,
 11. dynamische controle van de software op aanwezigheid van kwetsbare constructies,
@@ -437,7 +437,7 @@
 5. release van software: Releaseserver in het ontwikkelplatform,
 6. maken van testrapportages: JUnit, Robot Framework, TestNG, of hiermee compatible tools,
 7. maken van kwaliteitsrapportages: Quality-time,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),
+8. actueel houden van externe software: RenovateBot,
 9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,
 10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,
 11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,
@@ -1114,7 +1114,7 @@
     <t>7. maken van kwaliteitsrapportages: Quality-time,</t>
   </si>
   <si>
-    <t>8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),</t>
+    <t>8. actueel houden van externe software: RenovateBot,</t>
   </si>
   <si>
     <t>9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,</t>

</xml_diff>

<commit_message>
Voeg kennis van KA toe aan M23.
De titel van maatregel M23 is veranderd van "Het project zorgt voor de aanwezigheid van ervaring met de Kwaliteitsaanpak" naar "Het project zorgt voor de aanwezigheid van kennis van en ervaring met de Kwaliteitsaanpak". Aan de inhoud is toegevoegd dat nieuwe projectleden uitleg over de Kwaliteitsaanpak krijgen.

Closes #794.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -417,17 +417,16 @@
 5. release van software,
 6. maken van testrapportages,
 7. maken van kwaliteitsrapportages,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden,
-9. controleren van door de applicatie gebruikte versies van externe software op aanwezigheid van bekende kwetsbaarheden,
-10. statische controle van de software op aanwezigheid van kwetsbare constructies,
-11. dynamische controle van de software op aanwezigheid van kwetsbare constructies,
-12. controleren van container images op aanwezigheid van bekende kwetsbaarheden,
-13. testen van performance en schaalbaarheid,
-14. testen op toegankelijkheid van de applicatie,
-15. produceren van een "software bill of materials" (SBoM),
-16. opslaan van artifacten,
-17. registratie van incidenten bij gebruik en beheer, en
-18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving.
+8. controleren van door de applicatie gebruikte versies van externe software op aanwezigheid van bekende kwetsbaarheden,
+9. statische controle van de software op aanwezigheid van kwetsbare constructies,
+10. dynamische controle van de software op aanwezigheid van kwetsbare constructies,
+11. controleren van container images op aanwezigheid van bekende kwetsbaarheden,
+12. testen van performance en schaalbaarheid,
+13. testen op toegankelijkheid van de applicatie,
+14. produceren van een "software bill of materials" (SBoM),
+15. opslaan van artifacten,
+16. registratie van incidenten bij gebruik en beheer, en
+17. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving.
 Onder het ondersteunen van "agile werken" vallen het opvoeren van eisen, het opvoeren van logische testgevallen, het koppelen van logische testgevallen aan eisen, het bijhouden van een werkvoorraad, het plannen van iteraties en het toewijzen van eisen aan iteraties. De 'eisen' worden, conform Scrumterminologie, geregistreerd als epics en/of user stories, de werkvoorraad als product backlog en de iteraties als sprints. Het toewijzen van eisen aan iteraties gebeurt via de sprint backlog.
 ICTU adviseert en ondersteunt voor de genoemde taken onderstaande tools. Projecten gebruiken deze tools, of gelijkwaardige alternatieven:
 1. product en sprint backlog management en agile werken: Azure DevOps of Jira,
@@ -437,17 +436,16 @@
 5. release van software: Releaseserver in het ontwikkelplatform,
 6. maken van testrapportages: JUnit, Robot Framework, TestNG, of hiermee compatible tools,
 7. maken van kwaliteitsrapportages: Quality-time,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),
-9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,
-10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,
-11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,
-12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,
-13. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,
-14. testen op toegankelijkheid van de applicatie: Axe,
-15. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,
-16. opslaan van artifacten: Nexus of Harbor,
-17. registratie van incidenten bij gebruik en beheer: Jira, en
-18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.
+8. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,
+9. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,
+10. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,
+11. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,
+12. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,
+13. testen op toegankelijkheid van de applicatie: Axe,
+14. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,
+15. opslaan van artifacten: Nexus of Harbor,
+16. registratie van incidenten bij gebruik en beheer: Jira, en
+17. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.
 Rationale
 Projecten hebben een redelijke vrijheid bij het kiezen en gebruiken van tools, maar voor een aantal taken is het gebruik verplicht gesteld. Deze tools zijn nodig voor een efficiënte uitvoering van de Kwaliteitsaanpak. Uniform gebruik van deze tools maakt het mogelijk koppeling tussen die tools voor alle projecten te standaardiseren; daarnaast bevordert het de uitwisselbaarheid van medewerkers en neemt het risico op het gebruik van onvolwassen tools af. Tot slot is het gebruik in een aantal gevallen, ten behoeve van informatiebeveiliging bij de overheid, verplicht.
 </t>
@@ -467,7 +465,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B76" authorId="0">
+    <comment ref="B75" authorId="0">
       <text>
         <r>
           <rPr>
@@ -487,7 +485,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B77" authorId="0">
+    <comment ref="B76" authorId="0">
       <text>
         <r>
           <rPr>
@@ -509,7 +507,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B79" authorId="0">
+    <comment ref="B78" authorId="0">
       <text>
         <r>
           <rPr>
@@ -530,7 +528,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B80" authorId="0">
+    <comment ref="B79" authorId="0">
       <text>
         <r>
           <rPr>
@@ -547,7 +545,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B81" authorId="0">
+    <comment ref="B80" authorId="0">
       <text>
         <r>
           <rPr>
@@ -556,15 +554,15 @@
             <rFont val="Courier"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">M23: Het project zorgt voor de aanwezigheid van ervaring met de Kwaliteitsaanpak
-De software delivery manager zorgt ervoor dat bij nieuwe projecten wordt gestart met ten minste twee projectleden die bekend zijn met de Kwaliteitsaanpak.
+          <t xml:space="preserve">M23: Het project zorgt voor de aanwezigheid van kennis van en ervaring met de Kwaliteitsaanpak
+De software delivery manager zorgt ervoor dat bij nieuwe projecten wordt gestart met ten minste twee projectleden die bekend zijn met de Kwaliteitsaanpak. Projectleden die nog niet bekend zijn met de Kwaliteitsaanpak krijgen uitleg over de inhoud en achtergrond van de Kwaliteitsaanpak.
 Rationale
 Het inzetten van teamleden die bekend zijn met de Kwaliteitsaanpak zorgt voor een soepeler start van een nieuw project omdat zij bekend zijn met de inhoud van de Kwaliteitsaanpak, zoals kwaliteitsnormen en tools, en omdat zij al doende nieuwe teamleden bekend kunnen maken met de Kwaliteitsaanpak.
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="B82" authorId="0">
+    <comment ref="B81" authorId="0">
       <text>
         <r>
           <rPr>
@@ -587,7 +585,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C82" authorId="0">
+    <comment ref="C81" authorId="0">
       <text>
         <r>
           <rPr>
@@ -600,7 +598,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B87" authorId="0">
+    <comment ref="B86" authorId="0">
       <text>
         <r>
           <rPr>
@@ -621,7 +619,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B88" authorId="0">
+    <comment ref="B87" authorId="0">
       <text>
         <r>
           <rPr>
@@ -646,7 +644,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B89" authorId="0">
+    <comment ref="B88" authorId="0">
       <text>
         <r>
           <rPr>
@@ -673,7 +671,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B90" authorId="0">
+    <comment ref="B89" authorId="0">
       <text>
         <r>
           <rPr>
@@ -691,7 +689,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B91" authorId="0">
+    <comment ref="B90" authorId="0">
       <text>
         <r>
           <rPr>
@@ -723,7 +721,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C91" authorId="0">
+    <comment ref="C90" authorId="0">
       <text>
         <r>
           <rPr>
@@ -736,7 +734,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B106" authorId="0">
+    <comment ref="B105" authorId="0">
       <text>
         <r>
           <rPr>
@@ -756,7 +754,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B108" authorId="0">
+    <comment ref="B107" authorId="0">
       <text>
         <r>
           <rPr>
@@ -776,7 +774,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B109" authorId="0">
+    <comment ref="B108" authorId="0">
       <text>
         <r>
           <rPr>
@@ -795,7 +793,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B110" authorId="0">
+    <comment ref="B109" authorId="0">
       <text>
         <r>
           <rPr>
@@ -816,7 +814,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B111" authorId="0">
+    <comment ref="B110" authorId="0">
       <text>
         <r>
           <rPr>
@@ -835,7 +833,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B112" authorId="0">
+    <comment ref="B111" authorId="0">
       <text>
         <r>
           <rPr>
@@ -853,7 +851,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B113" authorId="0">
+    <comment ref="B112" authorId="0">
       <text>
         <r>
           <rPr>
@@ -884,9 +882,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
-  <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 04-03-2025.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="145">
+  <si>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 21-03-2025.</t>
   </si>
   <si>
     <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Bij maatregelen met submaatregelen hoeft alleen de status van de submaatregelen te worden ingevuld.</t>
@@ -1114,37 +1112,34 @@
     <t>7. maken van kwaliteitsrapportages: Quality-time,</t>
   </si>
   <si>
-    <t>8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),</t>
-  </si>
-  <si>
-    <t>9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,</t>
-  </si>
-  <si>
-    <t>10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,</t>
-  </si>
-  <si>
-    <t>11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,</t>
-  </si>
-  <si>
-    <t>12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,</t>
-  </si>
-  <si>
-    <t>13. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,</t>
-  </si>
-  <si>
-    <t>14. testen op toegankelijkheid van de applicatie: Axe,</t>
-  </si>
-  <si>
-    <t>15. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,</t>
-  </si>
-  <si>
-    <t>16. opslaan van artifacten: Nexus of Harbor,</t>
-  </si>
-  <si>
-    <t>17. registratie van incidenten bij gebruik en beheer: Jira, en</t>
-  </si>
-  <si>
-    <t>18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.</t>
+    <t>8. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,</t>
+  </si>
+  <si>
+    <t>9. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,</t>
+  </si>
+  <si>
+    <t>10. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,</t>
+  </si>
+  <si>
+    <t>11. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,</t>
+  </si>
+  <si>
+    <t>12. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,</t>
+  </si>
+  <si>
+    <t>13. testen op toegankelijkheid van de applicatie: Axe,</t>
+  </si>
+  <si>
+    <t>14. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,</t>
+  </si>
+  <si>
+    <t>15. opslaan van artifacten: Nexus of Harbor,</t>
+  </si>
+  <si>
+    <t>16. registratie van incidenten bij gebruik en beheer: Jira, en</t>
+  </si>
+  <si>
+    <t>17. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.</t>
   </si>
   <si>
     <t>M08</t>
@@ -1177,7 +1172,7 @@
     <t>M23</t>
   </si>
   <si>
-    <t>Het project zorgt voor de aanwezigheid van ervaring met de Kwaliteitsaanpak</t>
+    <t>Het project zorgt voor de aanwezigheid van kennis van en ervaring met de Kwaliteitsaanpak</t>
   </si>
   <si>
     <t>M05</t>
@@ -1752,7 +1747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2378,79 +2373,79 @@
       <c r="D74" s="5"/>
     </row>
     <row r="75" spans="1:4">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6" t="s">
+      <c r="A75" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C75" s="7"/>
+      <c r="B75" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C75" s="4"/>
       <c r="D75" s="5"/>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C76" s="4"/>
       <c r="D76" s="5"/>
     </row>
     <row r="77" spans="1:4">
-      <c r="A77" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B77" s="3" t="s">
+      <c r="A77" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C77" s="4"/>
-      <c r="D77" s="5"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="1" t="s">
+      <c r="A78" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
-      <c r="D78" s="1"/>
+      <c r="B78" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C78" s="4"/>
+      <c r="D78" s="5"/>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C79" s="4"/>
       <c r="D79" s="5"/>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C80" s="4"/>
       <c r="D80" s="5"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C81" s="4"/>
       <c r="D81" s="5"/>
     </row>
     <row r="82" spans="1:4">
-      <c r="A82" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B82" s="3" t="s">
+      <c r="A82" s="6"/>
+      <c r="B82" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C82" s="4"/>
+      <c r="C82" s="7"/>
       <c r="D82" s="5"/>
     </row>
     <row r="83" spans="1:4">
@@ -2478,61 +2473,61 @@
       <c r="D85" s="5"/>
     </row>
     <row r="86" spans="1:4">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6" t="s">
+      <c r="A86" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C86" s="7"/>
+      <c r="B86" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C86" s="4"/>
       <c r="D86" s="5"/>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C87" s="4"/>
       <c r="D87" s="5"/>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C88" s="4"/>
       <c r="D88" s="5"/>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C89" s="4"/>
       <c r="D89" s="5"/>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C90" s="4"/>
       <c r="D90" s="5"/>
     </row>
     <row r="91" spans="1:4">
-      <c r="A91" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B91" s="3" t="s">
+      <c r="A91" s="6"/>
+      <c r="B91" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C91" s="4"/>
+      <c r="C91" s="7"/>
       <c r="D91" s="5"/>
     </row>
     <row r="92" spans="1:4">
@@ -2640,90 +2635,82 @@
       <c r="D104" s="5"/>
     </row>
     <row r="105" spans="1:4">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6" t="s">
+      <c r="A105" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C105" s="7"/>
+      <c r="B105" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C105" s="4"/>
       <c r="D105" s="5"/>
     </row>
     <row r="106" spans="1:4">
-      <c r="A106" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B106" s="3" t="s">
+      <c r="A106" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C106" s="4"/>
-      <c r="D106" s="5"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
     </row>
     <row r="107" spans="1:4">
-      <c r="A107" s="1" t="s">
+      <c r="A107" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
-      <c r="D107" s="1"/>
+      <c r="B107" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C107" s="4"/>
+      <c r="D107" s="5"/>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C108" s="4"/>
       <c r="D108" s="5"/>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C109" s="4"/>
       <c r="D109" s="5"/>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C110" s="4"/>
       <c r="D110" s="5"/>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C111" s="4"/>
       <c r="D111" s="5"/>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C112" s="4"/>
       <c r="D112" s="5"/>
-    </row>
-    <row r="113" spans="1:4">
-      <c r="A113" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C113" s="4"/>
-      <c r="D113" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2830,7 +2817,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C106">
+  <conditionalFormatting sqref="C107">
     <cfRule type="cellIs" dxfId="0" priority="393" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2928,20 +2915,6 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C113">
-    <cfRule type="cellIs" dxfId="0" priority="417" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="418" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="419" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="420" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C12">
     <cfRule type="cellIs" dxfId="0" priority="21" operator="equal">
       <formula>"voldoet"</formula>
@@ -3866,7 +3839,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C77">
+  <conditionalFormatting sqref="C78">
     <cfRule type="cellIs" dxfId="0" priority="281" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4202,7 +4175,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="105">
+  <dataValidations count="104">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4413,7 +4386,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C76">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C77">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C78">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C79">
@@ -4497,7 +4470,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C105">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C106">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C107">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C108">
@@ -4513,9 +4486,6 @@
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C112">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C113">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4537,7 +4507,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4545,10 +4515,10 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>145</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
M13 over ISO-25010 is vervallen.
Maatregel M13 "Het project gebruikt ISO-25010 voor de specificatie van productkwaliteitseisen" is vervallen. Het gebruik van ISO-25010 voor de specificatie van productkwaliteitseisen staat al genoemd in M01 "Het project levert in elke fase vastgestelde producten en informatie op".

Closes #950.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -290,24 +290,6 @@
             <rFont val="Courier"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">M13: Het project gebruikt ISO-25010 voor de specificatie van productkwaliteitseisen
-Voor specificatie en documentatie van vereiste en gewenste kwaliteitseigenschappen, de niet-functionele eisen, maken projecten gebruik van de terminologie en categorisering uit NEN-ISO/IEC 25010:2023. Projecten gebruiken NEN-ISO/IEC 25010:2023 om te controleren of alle relevante kwaliteitseigenschappen van het op te leveren eindproduct worden meegenomen in de ontwikkeling en/of onderhoud van het product.
-De standaard NEN-ISO/IEC 25010:2023 biedt een model voor het beschrijven van productkwaliteit. Kwaliteitseigenschappen zijn voorzien van een naam, definitie en classificatie. NEN-ISO/IEC 25010:2023 dekt een breed spectrum van kwaliteitseigenschappen af.
-Rationale
-NEN-ISO/IEC 25010:2023 biedt een model voor productkwaliteit. De standaard biedt geen concrete maatregelen, maar biedt wel een begrippenkader en dekt het volledige spectrum van mogelijk relevante kwaliteitseigenschappen af. Het gebruiken van een standaard voor specificatie van kwaliteit voorkomt miscommunicatie over kwaliteitseigenschappen en de breedte van de standaard zorgt ervoor dat alle relevante aspecten aan bod komen.
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B41" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Courier"/>
-            <family val="2"/>
-          </rPr>
           <t xml:space="preserve">M04: Het project borgt de correcte werking van het product met geautomatiseerde regressietests
 Regressietests - tests die verifiëren of eerder ontwikkelde software nog steeds correct werkt na wijzigingen in de software of aansluiting op andere externe koppelvlakken - zijn geautomatiseerd.
 Het project hanteert een norm voor de dekking van regressietests, legt deze vast in Quality-time en bewaakt deze.
@@ -317,7 +299,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B42" authorId="0">
+    <comment ref="B41" authorId="0">
       <text>
         <r>
           <rPr>
@@ -346,7 +328,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C42" authorId="0">
+    <comment ref="C41" authorId="0">
       <text>
         <r>
           <rPr>
@@ -359,7 +341,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B52" authorId="0">
+    <comment ref="B51" authorId="0">
       <text>
         <r>
           <rPr>
@@ -396,7 +378,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C52" authorId="0">
+    <comment ref="C51" authorId="0">
       <text>
         <r>
           <rPr>
@@ -409,7 +391,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B70" authorId="0">
+    <comment ref="B69" authorId="0">
       <text>
         <r>
           <rPr>
@@ -429,7 +411,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B71" authorId="0">
+    <comment ref="B70" authorId="0">
       <text>
         <r>
           <rPr>
@@ -451,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B73" authorId="0">
+    <comment ref="B72" authorId="0">
       <text>
         <r>
           <rPr>
@@ -472,7 +454,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B74" authorId="0">
+    <comment ref="B73" authorId="0">
       <text>
         <r>
           <rPr>
@@ -489,7 +471,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B75" authorId="0">
+    <comment ref="B74" authorId="0">
       <text>
         <r>
           <rPr>
@@ -506,7 +488,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B76" authorId="0">
+    <comment ref="B75" authorId="0">
       <text>
         <r>
           <rPr>
@@ -529,7 +511,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C76" authorId="0">
+    <comment ref="C75" authorId="0">
       <text>
         <r>
           <rPr>
@@ -542,7 +524,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B81" authorId="0">
+    <comment ref="B80" authorId="0">
       <text>
         <r>
           <rPr>
@@ -563,7 +545,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B82" authorId="0">
+    <comment ref="B81" authorId="0">
       <text>
         <r>
           <rPr>
@@ -588,7 +570,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B83" authorId="0">
+    <comment ref="B82" authorId="0">
       <text>
         <r>
           <rPr>
@@ -615,7 +597,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B84" authorId="0">
+    <comment ref="B83" authorId="0">
       <text>
         <r>
           <rPr>
@@ -633,7 +615,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B85" authorId="0">
+    <comment ref="B84" authorId="0">
       <text>
         <r>
           <rPr>
@@ -665,7 +647,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C85" authorId="0">
+    <comment ref="C84" authorId="0">
       <text>
         <r>
           <rPr>
@@ -678,7 +660,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B100" authorId="0">
+    <comment ref="B99" authorId="0">
       <text>
         <r>
           <rPr>
@@ -698,7 +680,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B102" authorId="0">
+    <comment ref="B101" authorId="0">
       <text>
         <r>
           <rPr>
@@ -718,7 +700,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B103" authorId="0">
+    <comment ref="B102" authorId="0">
       <text>
         <r>
           <rPr>
@@ -737,7 +719,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B104" authorId="0">
+    <comment ref="B103" authorId="0">
       <text>
         <r>
           <rPr>
@@ -758,7 +740,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B105" authorId="0">
+    <comment ref="B104" authorId="0">
       <text>
         <r>
           <rPr>
@@ -777,7 +759,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B106" authorId="0">
+    <comment ref="B105" authorId="0">
       <text>
         <r>
           <rPr>
@@ -795,7 +777,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B107" authorId="0">
+    <comment ref="B106" authorId="0">
       <text>
         <r>
           <rPr>
@@ -826,7 +808,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="137">
   <si>
     <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 24-03-2025.</t>
   </si>
@@ -964,12 +946,6 @@
   </si>
   <si>
     <t>Het project zorgt dat het product traceerbaar aan eisen voldoet</t>
-  </si>
-  <si>
-    <t>M13</t>
-  </si>
-  <si>
-    <t>Het project gebruikt ISO-25010 voor de specificatie van productkwaliteitseisen</t>
   </si>
   <si>
     <t>M04</t>
@@ -1684,7 +1660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D107"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2036,23 +2012,21 @@
       <c r="B41" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C41" s="8"/>
+      <c r="C41" s="4"/>
       <c r="D41" s="5"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C42" s="4"/>
+      <c r="C42" s="7"/>
       <c r="D42" s="5"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="6"/>
       <c r="B43" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C43" s="7"/>
       <c r="D43" s="5"/>
@@ -2060,7 +2034,7 @@
     <row r="44" spans="1:4">
       <c r="A44" s="6"/>
       <c r="B44" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="5"/>
@@ -2068,7 +2042,7 @@
     <row r="45" spans="1:4">
       <c r="A45" s="6"/>
       <c r="B45" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="5"/>
@@ -2076,7 +2050,7 @@
     <row r="46" spans="1:4">
       <c r="A46" s="6"/>
       <c r="B46" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="5"/>
@@ -2084,7 +2058,7 @@
     <row r="47" spans="1:4">
       <c r="A47" s="6"/>
       <c r="B47" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="5"/>
@@ -2092,7 +2066,7 @@
     <row r="48" spans="1:4">
       <c r="A48" s="6"/>
       <c r="B48" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="5"/>
@@ -2100,7 +2074,7 @@
     <row r="49" spans="1:4">
       <c r="A49" s="6"/>
       <c r="B49" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="5"/>
@@ -2108,33 +2082,33 @@
     <row r="50" spans="1:4">
       <c r="A50" s="6"/>
       <c r="B50" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C50" s="7"/>
       <c r="D50" s="5"/>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6" t="s">
+      <c r="A51" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C51" s="7"/>
+      <c r="C51" s="4"/>
       <c r="D51" s="5"/>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="6"/>
+      <c r="B52" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C52" s="4"/>
+      <c r="C52" s="7"/>
       <c r="D52" s="5"/>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="6"/>
       <c r="B53" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C53" s="7"/>
       <c r="D53" s="5"/>
@@ -2142,7 +2116,7 @@
     <row r="54" spans="1:4">
       <c r="A54" s="6"/>
       <c r="B54" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C54" s="7"/>
       <c r="D54" s="5"/>
@@ -2150,7 +2124,7 @@
     <row r="55" spans="1:4">
       <c r="A55" s="6"/>
       <c r="B55" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C55" s="7"/>
       <c r="D55" s="5"/>
@@ -2158,7 +2132,7 @@
     <row r="56" spans="1:4">
       <c r="A56" s="6"/>
       <c r="B56" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C56" s="7"/>
       <c r="D56" s="5"/>
@@ -2166,7 +2140,7 @@
     <row r="57" spans="1:4">
       <c r="A57" s="6"/>
       <c r="B57" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C57" s="7"/>
       <c r="D57" s="5"/>
@@ -2174,7 +2148,7 @@
     <row r="58" spans="1:4">
       <c r="A58" s="6"/>
       <c r="B58" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C58" s="7"/>
       <c r="D58" s="5"/>
@@ -2182,7 +2156,7 @@
     <row r="59" spans="1:4">
       <c r="A59" s="6"/>
       <c r="B59" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C59" s="7"/>
       <c r="D59" s="5"/>
@@ -2190,7 +2164,7 @@
     <row r="60" spans="1:4">
       <c r="A60" s="6"/>
       <c r="B60" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C60" s="7"/>
       <c r="D60" s="5"/>
@@ -2198,7 +2172,7 @@
     <row r="61" spans="1:4">
       <c r="A61" s="6"/>
       <c r="B61" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C61" s="7"/>
       <c r="D61" s="5"/>
@@ -2206,7 +2180,7 @@
     <row r="62" spans="1:4">
       <c r="A62" s="6"/>
       <c r="B62" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C62" s="7"/>
       <c r="D62" s="5"/>
@@ -2214,7 +2188,7 @@
     <row r="63" spans="1:4">
       <c r="A63" s="6"/>
       <c r="B63" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C63" s="7"/>
       <c r="D63" s="5"/>
@@ -2222,7 +2196,7 @@
     <row r="64" spans="1:4">
       <c r="A64" s="6"/>
       <c r="B64" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C64" s="7"/>
       <c r="D64" s="5"/>
@@ -2230,7 +2204,7 @@
     <row r="65" spans="1:4">
       <c r="A65" s="6"/>
       <c r="B65" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C65" s="7"/>
       <c r="D65" s="5"/>
@@ -2238,7 +2212,7 @@
     <row r="66" spans="1:4">
       <c r="A66" s="6"/>
       <c r="B66" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C66" s="7"/>
       <c r="D66" s="5"/>
@@ -2246,7 +2220,7 @@
     <row r="67" spans="1:4">
       <c r="A67" s="6"/>
       <c r="B67" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="7"/>
       <c r="D67" s="5"/>
@@ -2254,17 +2228,19 @@
     <row r="68" spans="1:4">
       <c r="A68" s="6"/>
       <c r="B68" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="5"/>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6" t="s">
+      <c r="A69" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B69" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C69" s="7"/>
+      <c r="C69" s="8"/>
       <c r="D69" s="5"/>
     </row>
     <row r="70" spans="1:4">
@@ -2278,22 +2254,22 @@
       <c r="D70" s="5"/>
     </row>
     <row r="71" spans="1:4">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C71" s="8"/>
-      <c r="D71" s="5"/>
-    </row>
-    <row r="72" spans="1:4">
-      <c r="A72" s="1" t="s">
+      <c r="B72" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="D72" s="1"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="5"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="3" t="s">
@@ -2322,23 +2298,21 @@
       <c r="B75" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C75" s="8"/>
+      <c r="C75" s="4"/>
       <c r="D75" s="5"/>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="3" t="s">
+      <c r="A76" s="6"/>
+      <c r="B76" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B76" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C76" s="4"/>
+      <c r="C76" s="7"/>
       <c r="D76" s="5"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="6"/>
       <c r="B77" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C77" s="7"/>
       <c r="D77" s="5"/>
@@ -2346,7 +2320,7 @@
     <row r="78" spans="1:4">
       <c r="A78" s="6"/>
       <c r="B78" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C78" s="7"/>
       <c r="D78" s="5"/>
@@ -2354,17 +2328,19 @@
     <row r="79" spans="1:4">
       <c r="A79" s="6"/>
       <c r="B79" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C79" s="7"/>
       <c r="D79" s="5"/>
     </row>
     <row r="80" spans="1:4">
-      <c r="A80" s="6"/>
-      <c r="B80" s="6" t="s">
+      <c r="A80" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B80" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C80" s="7"/>
+      <c r="C80" s="8"/>
       <c r="D80" s="5"/>
     </row>
     <row r="81" spans="1:4">
@@ -2404,23 +2380,21 @@
       <c r="B84" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C84" s="8"/>
+      <c r="C84" s="4"/>
       <c r="D84" s="5"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="3" t="s">
+      <c r="A85" s="6"/>
+      <c r="B85" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B85" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C85" s="4"/>
+      <c r="C85" s="7"/>
       <c r="D85" s="5"/>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="6"/>
       <c r="B86" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C86" s="7"/>
       <c r="D86" s="5"/>
@@ -2428,7 +2402,7 @@
     <row r="87" spans="1:4">
       <c r="A87" s="6"/>
       <c r="B87" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C87" s="7"/>
       <c r="D87" s="5"/>
@@ -2436,7 +2410,7 @@
     <row r="88" spans="1:4">
       <c r="A88" s="6"/>
       <c r="B88" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C88" s="7"/>
       <c r="D88" s="5"/>
@@ -2444,7 +2418,7 @@
     <row r="89" spans="1:4">
       <c r="A89" s="6"/>
       <c r="B89" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C89" s="7"/>
       <c r="D89" s="5"/>
@@ -2452,7 +2426,7 @@
     <row r="90" spans="1:4">
       <c r="A90" s="6"/>
       <c r="B90" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C90" s="7"/>
       <c r="D90" s="5"/>
@@ -2460,7 +2434,7 @@
     <row r="91" spans="1:4">
       <c r="A91" s="6"/>
       <c r="B91" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C91" s="7"/>
       <c r="D91" s="5"/>
@@ -2468,7 +2442,7 @@
     <row r="92" spans="1:4">
       <c r="A92" s="6"/>
       <c r="B92" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C92" s="7"/>
       <c r="D92" s="5"/>
@@ -2476,7 +2450,7 @@
     <row r="93" spans="1:4">
       <c r="A93" s="6"/>
       <c r="B93" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C93" s="7"/>
       <c r="D93" s="5"/>
@@ -2484,7 +2458,7 @@
     <row r="94" spans="1:4">
       <c r="A94" s="6"/>
       <c r="B94" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C94" s="7"/>
       <c r="D94" s="5"/>
@@ -2492,7 +2466,7 @@
     <row r="95" spans="1:4">
       <c r="A95" s="6"/>
       <c r="B95" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C95" s="7"/>
       <c r="D95" s="5"/>
@@ -2500,7 +2474,7 @@
     <row r="96" spans="1:4">
       <c r="A96" s="6"/>
       <c r="B96" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C96" s="7"/>
       <c r="D96" s="5"/>
@@ -2508,7 +2482,7 @@
     <row r="97" spans="1:4">
       <c r="A97" s="6"/>
       <c r="B97" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C97" s="7"/>
       <c r="D97" s="5"/>
@@ -2516,36 +2490,38 @@
     <row r="98" spans="1:4">
       <c r="A98" s="6"/>
       <c r="B98" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C98" s="7"/>
       <c r="D98" s="5"/>
     </row>
     <row r="99" spans="1:4">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6" t="s">
+      <c r="A99" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B99" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C99" s="7"/>
+      <c r="C99" s="8"/>
       <c r="D99" s="5"/>
     </row>
     <row r="100" spans="1:4">
-      <c r="A100" s="3" t="s">
+      <c r="A100" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C100" s="8"/>
-      <c r="D100" s="5"/>
-    </row>
-    <row r="101" spans="1:4">
-      <c r="A101" s="1" t="s">
+      <c r="B101" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
+      <c r="C101" s="8"/>
+      <c r="D101" s="5"/>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="3" t="s">
@@ -2596,16 +2572,6 @@
       </c>
       <c r="C106" s="8"/>
       <c r="D106" s="5"/>
-    </row>
-    <row r="107" spans="1:4">
-      <c r="A107" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C107" s="8"/>
-      <c r="D107" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2628,7 +2594,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C100">
+  <conditionalFormatting sqref="C101">
     <cfRule type="cellIs" dxfId="0" priority="341" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2712,20 +2678,6 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C107">
-    <cfRule type="cellIs" dxfId="0" priority="365" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="366" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="367" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="368" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C11">
     <cfRule type="cellIs" dxfId="0" priority="13" operator="equal">
       <formula>"voldoet"</formula>
@@ -3118,7 +3070,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C41">
+  <conditionalFormatting sqref="C42">
     <cfRule type="cellIs" dxfId="0" priority="125" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3244,7 +3196,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C51">
+  <conditionalFormatting sqref="C52">
     <cfRule type="cellIs" dxfId="0" priority="161" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3510,7 +3462,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C71">
+  <conditionalFormatting sqref="C72">
     <cfRule type="cellIs" dxfId="0" priority="237" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3552,7 +3504,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C75">
+  <conditionalFormatting sqref="C76">
     <cfRule type="cellIs" dxfId="0" priority="249" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3678,7 +3630,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C84">
+  <conditionalFormatting sqref="C85">
     <cfRule type="cellIs" dxfId="0" priority="281" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3902,7 +3854,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="92">
+  <dataValidations count="91">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -3996,7 +3948,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C40">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C41">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C42">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C43">
@@ -4023,7 +3975,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C50">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C51">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C52">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C53">
@@ -4080,7 +4032,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C70">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C71">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C72">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C73">
@@ -4089,7 +4041,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C74">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C75">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C76">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C77">
@@ -4113,7 +4065,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C83">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C84">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C85">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C86">
@@ -4158,7 +4110,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C99">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C100">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C101">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C102">
@@ -4174,9 +4126,6 @@
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C106">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C107">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4185,31 +4134,30 @@
     <hyperlink ref="A28" r:id="rId2" location="m32"/>
     <hyperlink ref="A32" r:id="rId3" location="m02"/>
     <hyperlink ref="A39" r:id="rId4" location="m03"/>
-    <hyperlink ref="A40" r:id="rId5" location="m13"/>
-    <hyperlink ref="A41" r:id="rId6" location="m04"/>
-    <hyperlink ref="A42" r:id="rId7" location="m07"/>
-    <hyperlink ref="A52" r:id="rId8" location="m16"/>
-    <hyperlink ref="A70" r:id="rId9" location="m08"/>
-    <hyperlink ref="A71" r:id="rId10" location="m26"/>
-    <hyperlink ref="A73" r:id="rId11" location="m14"/>
-    <hyperlink ref="A74" r:id="rId12" location="m21"/>
-    <hyperlink ref="A75" r:id="rId13" location="m23"/>
-    <hyperlink ref="A76" r:id="rId14" location="m05"/>
-    <hyperlink ref="A81" r:id="rId15" location="m35"/>
-    <hyperlink ref="A82" r:id="rId16" location="m10"/>
-    <hyperlink ref="A83" r:id="rId17" location="m28"/>
-    <hyperlink ref="A84" r:id="rId18" location="m30"/>
-    <hyperlink ref="A85" r:id="rId19" location="m34"/>
-    <hyperlink ref="A100" r:id="rId20" location="m27"/>
-    <hyperlink ref="A102" r:id="rId21" location="m29"/>
-    <hyperlink ref="A103" r:id="rId22" location="m19"/>
-    <hyperlink ref="A104" r:id="rId23" location="m18"/>
-    <hyperlink ref="A105" r:id="rId24" location="m11"/>
-    <hyperlink ref="A106" r:id="rId25" location="m12"/>
-    <hyperlink ref="A107" r:id="rId26" location="m33"/>
+    <hyperlink ref="A40" r:id="rId5" location="m04"/>
+    <hyperlink ref="A41" r:id="rId6" location="m07"/>
+    <hyperlink ref="A51" r:id="rId7" location="m16"/>
+    <hyperlink ref="A69" r:id="rId8" location="m08"/>
+    <hyperlink ref="A70" r:id="rId9" location="m26"/>
+    <hyperlink ref="A72" r:id="rId10" location="m14"/>
+    <hyperlink ref="A73" r:id="rId11" location="m21"/>
+    <hyperlink ref="A74" r:id="rId12" location="m23"/>
+    <hyperlink ref="A75" r:id="rId13" location="m05"/>
+    <hyperlink ref="A80" r:id="rId14" location="m35"/>
+    <hyperlink ref="A81" r:id="rId15" location="m10"/>
+    <hyperlink ref="A82" r:id="rId16" location="m28"/>
+    <hyperlink ref="A83" r:id="rId17" location="m30"/>
+    <hyperlink ref="A84" r:id="rId18" location="m34"/>
+    <hyperlink ref="A99" r:id="rId19" location="m27"/>
+    <hyperlink ref="A101" r:id="rId20" location="m29"/>
+    <hyperlink ref="A102" r:id="rId21" location="m19"/>
+    <hyperlink ref="A103" r:id="rId22" location="m18"/>
+    <hyperlink ref="A104" r:id="rId23" location="m11"/>
+    <hyperlink ref="A105" r:id="rId24" location="m12"/>
+    <hyperlink ref="A106" r:id="rId25" location="m33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId27"/>
+  <legacyDrawing r:id="rId26"/>
 </worksheet>
 </file>
 
@@ -4226,7 +4174,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4234,10 +4182,10 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
In M16 de twee opsommingen gecombineerd in 1 tabel.
In M16 "Het project gebruikt tools voor vastgestelde taken" de opsomming van taken gecombineerd met de opsomming van tools in één tabel.

Closes #937.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -374,12 +374,9 @@
 6. Toegankelijkheidstests,
 7. Broncodekwaliteitscontroles,
 8. Installatie van de software in test, acceptatie en/of productieomgevingen,
-9. Produceren van een "software bill of materials" (SBoM),
-10. Oplevering van het totale product, dus inclusief alle deliverables, in de vorm zoals bruikbaar voor en afgesproken met de opdrachtgevende organisatie.
+9. Oplevering van het totale product, dus inclusief alle deliverables, in de vorm zoals bruikbaar voor en afgesproken met de opdrachtgevende organisatie.
 Performance- en beveiligingstests op de software zijn ook onderdeel van de continuous delivery pipeline, maar vanwege doorlooptijden en licenties is dat niet altijd haalbaar; in dat geval vinden de performance- en beveiligingstests zo veel mogelijk, en bij voorkeur dagelijks, plaats. Performance- en beveiligingstests op de software vinden plaats in de testomgeving van het project. Als ICTU verantwoordelijk is voor het operationeel beheer laat ICTU de performance- en beveiligingstesten op de software (ook) uitvoeren in een productie-like omgeving.
 Niet alle testen en controles kunnen altijd geautomatiseerd worden uitgevoerd. Denk aan kwaliteitscontroles op architectuurbeslissingen of het testen van toegankelijkheidseisen. Waar mogelijk wordt wel een zo groot mogelijk deel van de testen en controles geautomatiseerd en als onderdeel van de pipeline uitgevoerd.
-De afdeling ICTU Software Diensten (ISD) voorziet in tools en ondersteuning, zodat projecten deze pipeline kunnen toepassen. Projecten zijn verantwoordelijk voor de correcte werking van de pipeline.
-ICTU gebruikt Jenkins, GitLab CI of Azure DevOps als tool voor de implementatie van de continuous delivery pipeline. ISD biedt de projecten een voorziening om releases van het totale product veilig op te leveren aan opdrachtgevende organisaties en beheerorganisaties.
 Rationale
 Software incrementeel opleveren vereist dat de software frequent gebouwd, getest en opgeleverd kan worden. Om dit efficiënt en foutvrij te doen, dient het proces van bouwen, testen en opleveren geautomatiseerd te zijn; een continuous delivery pipeline faciliteert dit.
 </t>
@@ -399,7 +396,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B57" authorId="0">
+    <comment ref="B56" authorId="0">
       <text>
         <r>
           <rPr>
@@ -409,52 +406,34 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">M16: Het project gebruikt tools voor vastgestelde taken
-ICTU stelt het gebruik van tools verplicht voor de volgende taken:
-1. product en sprint backlog management en agile werken,
-2. inrichten en uitvoeren van een continuous delivery pipeline,
-3. monitoren van de kwaliteit van broncode,
-4. versiebeheer van op te leveren producten,
-5. release van software,
-6. maken van testrapportages,
-7. maken van kwaliteitsrapportages,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden,
-9. controleren van door de applicatie gebruikte versies van externe software op aanwezigheid van bekende kwetsbaarheden,
-10. statische controle van de software op aanwezigheid van kwetsbare constructies,
-11. dynamische controle van de software op aanwezigheid van kwetsbare constructies,
-12. controleren van container images op aanwezigheid van bekende kwetsbaarheden,
-13. testen van performance en schaalbaarheid,
-14. testen op toegankelijkheid van de applicatie,
-15. produceren van een "software bill of materials" (SBoM),
-16. opslaan van artifacten,
-17. registratie van incidenten bij gebruik en beheer, en
-18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving.
-Onder het ondersteunen van "agile werken" vallen het opvoeren van eisen, het opvoeren van logische testgevallen, het koppelen van logische testgevallen aan eisen, het bijhouden van een werkvoorraad, het plannen van iteraties en het toewijzen van eisen aan iteraties. De 'eisen' worden, conform Scrumterminologie, geregistreerd als epics en/of user stories, de werkvoorraad als product backlog en de iteraties als sprints. Het toewijzen van eisen aan iteraties gebeurt via de sprint backlog.
-ICTU adviseert en ondersteunt voor de genoemde taken onderstaande tools. Projecten gebruiken deze tools, of gelijkwaardige alternatieven:
-1. product en sprint backlog management en agile werken: Azure DevOps of Jira,
-2. inrichten en uitvoeren van een continuous delivery pipeline: Jenkins, GitLab CI/CD (Continuous Integration, Delivery, and Deployment) of Azure DevOps,
-3. monitoren van de kwaliteit van broncode: SonarQube,
-4. versiebeheer van op te leveren producten: GitLab of Azure DevOps,
-5. release van software: Releaseserver in het ontwikkelplatform,
-6. maken van testrapportages: JUnit, Robot Framework, TestNG, of hiermee compatible tools,
-7. maken van kwaliteitsrapportages: Quality-time,
-8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),
-9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,
-10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,
-11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,
-12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,
-13. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,
-14. testen op toegankelijkheid van de applicatie: Axe,
-15. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,
-16. opslaan van artifacten: Nexus of Harbor,
-17. registratie van incidenten bij gebruik en beheer: Jira, en
-18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.
+Voor vastgestelde taken bij het ontwikkelen, onderhouden en operationeel beheren van software, stelt ICTU het gebruik van tools verplicht. ICTU adviseert per taak specifieke tools en ondersteunt projecten bij het gebruik daarvan.
+ICTU adviseert en ondersteunt voor de hieronder genoemde taken specifieke tools. Projecten gebruiken deze tools, of gelijkwaardige alternatieven.
+Activiteit                                                                                   Tools                                                                                    
+Product en sprint backlog management en agile werken                                         Azure DevOps of Jira                                                                     
+Inrichten en uitvoeren van een continuous delivery pipeline                                  Jenkins, GitLab CI/CD (Continuous Integration, Delivery, and Deployment) of Azure DevOps 
+Monitoren van de kwaliteit van broncode                                                      SonarQube                                                                                
+Versiebeheer van op te leveren producten                                                     GitLab of Azure DevOps                                                                   
+Release van software                                                                         Releaseserver in het ontwikkelplatform                                                   
+Maken van testrapportages                                                                    JUnit, Robot Framework, TestNG, of hiermee compatible tools                              
+Maken van kwaliteitsrapportages                                                              Quality-time                                                                             
+Controleren op aanwezigheid van bekende kwetsbaarheden in externe software                   OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track    
+Statische controle van de software op aanwezigheid van kwetsbare constructies                SonarQube                                                                                
+Dynamische controle van de software op aanwezigheid van kwetsbare constructies               ZAP (Zed Attack Proxy) by Checkmarx                                                      
+Controleren van container images op aanwezigheid van bekende kwetsbaarheden                  Trivy                                                                                    
+Testen van performance en schaalbaarheid                                                     JMeter en Performancetestrunner                                                          
+Testen op toegankelijkheid van de applicatie                                                 Axe                                                                                      
+Produceren van een "software bill of materials" (SBoM)                                       Tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren            
+Opslaan van artifacten                                                                       Nexus of Harbor                                                                          
+Registratie van incidenten bij gebruik en beheer                                             Jira                                                                                     
+Bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving Ansible                                                                                  
+N.B. Onder het ondersteunen van "agile werken" vallen het opvoeren van eisen, het opvoeren van logische testgevallen, het koppelen van logische testgevallen aan eisen, het bijhouden van een werkvoorraad, het plannen van iteraties en het toewijzen van eisen aan iteraties. De 'eisen' worden, conform Scrumterminologie, geregistreerd als epics en/of user stories, de werkvoorraad als product backlog en de iteraties als sprints. Het toewijzen van eisen aan iteraties gebeurt via de sprint backlog.
 Rationale
 Projecten hebben een redelijke vrijheid bij het kiezen en gebruiken van tools, maar voor een aantal taken is het gebruik verplicht gesteld. Deze tools zijn nodig voor een efficiënte uitvoering van de Kwaliteitsaanpak. Uniform gebruik van deze tools maakt het mogelijk koppeling tussen die tools voor alle projecten te standaardiseren; daarnaast bevordert het de uitwisselbaarheid van medewerkers en neemt het risico op het gebruik van onvolwassen tools af. Tot slot is het gebruik in een aantal gevallen, ten behoeve van informatiebeveiliging bij de overheid, verplicht.
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="C57" authorId="0">
+    <comment ref="C56" authorId="0">
       <text>
         <r>
           <rPr>
@@ -467,7 +446,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B76" authorId="0">
+    <comment ref="B74" authorId="0">
       <text>
         <r>
           <rPr>
@@ -487,7 +466,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B77" authorId="0">
+    <comment ref="B75" authorId="0">
       <text>
         <r>
           <rPr>
@@ -509,7 +488,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B79" authorId="0">
+    <comment ref="B77" authorId="0">
       <text>
         <r>
           <rPr>
@@ -530,7 +509,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B80" authorId="0">
+    <comment ref="B78" authorId="0">
       <text>
         <r>
           <rPr>
@@ -547,7 +526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B81" authorId="0">
+    <comment ref="B79" authorId="0">
       <text>
         <r>
           <rPr>
@@ -564,7 +543,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B82" authorId="0">
+    <comment ref="B80" authorId="0">
       <text>
         <r>
           <rPr>
@@ -587,7 +566,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C82" authorId="0">
+    <comment ref="C80" authorId="0">
       <text>
         <r>
           <rPr>
@@ -600,7 +579,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B87" authorId="0">
+    <comment ref="B85" authorId="0">
       <text>
         <r>
           <rPr>
@@ -621,7 +600,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B88" authorId="0">
+    <comment ref="B86" authorId="0">
       <text>
         <r>
           <rPr>
@@ -646,7 +625,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B89" authorId="0">
+    <comment ref="B87" authorId="0">
       <text>
         <r>
           <rPr>
@@ -673,7 +652,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B90" authorId="0">
+    <comment ref="B88" authorId="0">
       <text>
         <r>
           <rPr>
@@ -691,7 +670,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B91" authorId="0">
+    <comment ref="B89" authorId="0">
       <text>
         <r>
           <rPr>
@@ -723,7 +702,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C91" authorId="0">
+    <comment ref="C89" authorId="0">
       <text>
         <r>
           <rPr>
@@ -736,7 +715,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B106" authorId="0">
+    <comment ref="B104" authorId="0">
       <text>
         <r>
           <rPr>
@@ -756,7 +735,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B108" authorId="0">
+    <comment ref="B106" authorId="0">
       <text>
         <r>
           <rPr>
@@ -776,7 +755,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B109" authorId="0">
+    <comment ref="B107" authorId="0">
       <text>
         <r>
           <rPr>
@@ -795,7 +774,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B110" authorId="0">
+    <comment ref="B108" authorId="0">
       <text>
         <r>
           <rPr>
@@ -806,7 +785,7 @@
           </rPr>
           <t xml:space="preserve">M18: ICTU biedt ondersteuning voor verplicht gestelde tools
 ICTU zorgt voor technische en functionele ondersteuning aan projecten bij het gebruik van alle verplichte tools.
-ICTU zorgt voor ondersteuning van de bij M16: Het project gebruikt tools voor vastgestelde taken verplicht gestelde tools. Een team van specialisten met kennis, ervaring en capaciteit is beschikbaar voor ondersteuning aan projecten.
+ICTU zorgt voor ondersteuning van de in M16: Het project gebruikt tools voor vastgestelde taken verplicht gestelde tools. Een team van specialisten met kennis, ervaring en capaciteit is beschikbaar voor ondersteuning aan projecten. Projecten zijn verantwoordelijk voor de correcte werking van de pipeline.
 Bij de selectie van tools ter ondersteuning van de projectuitvoering geeft ICTU de voorkeur aan open source tools. Ook tools die ICTU zelf ontwikkelt ter ondersteuning van softwareontwikkelprojecten worden bij voorkeur open source beschikbaar gesteld.
 Rationale
 De keuze om het gebruik van een aantal tools verplicht te stellen (M16: Het project gebruikt tools voor vastgestelde taken) volgt uit de belangrijke rol die die tools spelen in de ontwikkelstraat en in Quality-time, het kwaliteitssysteem van ICTU. Met de verplichting komt ook een verantwoordelijkheid: om projecten in staat te stellen snel en effectief met deze tools te werken, moeten die projecten ondersteund worden.
@@ -816,7 +795,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B111" authorId="0">
+    <comment ref="B109" authorId="0">
       <text>
         <r>
           <rPr>
@@ -835,7 +814,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B112" authorId="0">
+    <comment ref="B110" authorId="0">
       <text>
         <r>
           <rPr>
@@ -853,7 +832,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B113" authorId="0">
+    <comment ref="B111" authorId="0">
       <text>
         <r>
           <rPr>
@@ -884,9 +863,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
-  <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 04-03-2025.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="144">
+  <si>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 21-03-2025.</t>
   </si>
   <si>
     <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Bij maatregelen met submaatregelen hoeft alleen de status van de submaatregelen te worden ingevuld.</t>
@@ -1081,10 +1060,7 @@
     <t>8. Installatie van de software in test, acceptatie en/of productieomgevingen,</t>
   </si>
   <si>
-    <t>9. Produceren van een "software bill of materials" (SBoM),</t>
-  </si>
-  <si>
-    <t>10. Oplevering van het totale product, dus inclusief alle deliverables, in de vorm zoals bruikbaar voor en afgesproken met de opdrachtgevende organisatie.</t>
+    <t>9. Oplevering van het totale product, dus inclusief alle deliverables, in de vorm zoals bruikbaar voor en afgesproken met de opdrachtgevende organisatie.</t>
   </si>
   <si>
     <t>M16</t>
@@ -1093,58 +1069,55 @@
     <t>Het project gebruikt tools voor vastgestelde taken</t>
   </si>
   <si>
-    <t>1. product en sprint backlog management en agile werken: Azure DevOps of Jira,</t>
-  </si>
-  <si>
-    <t>2. inrichten en uitvoeren van een continuous delivery pipeline: Jenkins, GitLab CI/CD (Continuous Integration, Delivery, and Deployment) of Azure DevOps,</t>
-  </si>
-  <si>
-    <t>3. monitoren van de kwaliteit van broncode: SonarQube,</t>
-  </si>
-  <si>
-    <t>4. versiebeheer van op te leveren producten: GitLab of Azure DevOps,</t>
-  </si>
-  <si>
-    <t>5. release van software: Releaseserver in het ontwikkelplatform,</t>
-  </si>
-  <si>
-    <t>6. maken van testrapportages: JUnit, Robot Framework, TestNG, of hiermee compatible tools,</t>
-  </si>
-  <si>
-    <t>7. maken van kwaliteitsrapportages: Quality-time,</t>
-  </si>
-  <si>
-    <t>8. controleren van de configuratie op aanwezigheid van bekende kwetsbaarheden in configuratie: OpenVAS (Vulnerability Assessment System),</t>
-  </si>
-  <si>
-    <t>9. controleren op aanwezigheid van bekende kwetsbaarheden in externe software: OWASP (Open Web Application Security Project) Dependency-Check en/of Dependency-Track,</t>
-  </si>
-  <si>
-    <t>10. statische controle van de software op aanwezigheid van kwetsbare constructies: SonarQube,</t>
-  </si>
-  <si>
-    <t>11. dynamische controle van de software op aanwezigheid van kwetsbare constructies: ZAP (Zed Attack Proxy) by Checkmarx,</t>
-  </si>
-  <si>
-    <t>12. controleren van container images op aanwezigheid van bekende kwetsbaarheden: Trivy,</t>
-  </si>
-  <si>
-    <t>13. testen van performance en schaalbaarheid: JMeter en Performancetestrunner,</t>
-  </si>
-  <si>
-    <t>14. testen op toegankelijkheid van de applicatie: Axe,</t>
-  </si>
-  <si>
-    <t>15. produceren van een "software bill of materials" (SBoM): tools die een SBoM in CycloneDX-formaat (zie https://cyclonedx.org) genereren,</t>
-  </si>
-  <si>
-    <t>16. opslaan van artifacten: Nexus of Harbor,</t>
-  </si>
-  <si>
-    <t>17. registratie van incidenten bij gebruik en beheer: Jira, en</t>
-  </si>
-  <si>
-    <t>18. bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving: Ansible.</t>
+    <t>1. Product en sprint backlog management en agile werken</t>
+  </si>
+  <si>
+    <t>2. Inrichten en uitvoeren van een continuous delivery pipeline</t>
+  </si>
+  <si>
+    <t>3. Monitoren van de kwaliteit van broncode</t>
+  </si>
+  <si>
+    <t>4. Versiebeheer van op te leveren producten</t>
+  </si>
+  <si>
+    <t>5. Release van software</t>
+  </si>
+  <si>
+    <t>6. Maken van testrapportages</t>
+  </si>
+  <si>
+    <t>7. Maken van kwaliteitsrapportages</t>
+  </si>
+  <si>
+    <t>8. Controleren op aanwezigheid van bekende kwetsbaarheden in externe software</t>
+  </si>
+  <si>
+    <t>9. Statische controle van de software op aanwezigheid van kwetsbare constructies</t>
+  </si>
+  <si>
+    <t>10. Dynamische controle van de software op aanwezigheid van kwetsbare constructies</t>
+  </si>
+  <si>
+    <t>11. Controleren van container images op aanwezigheid van bekende kwetsbaarheden</t>
+  </si>
+  <si>
+    <t>12. Testen van performance en schaalbaarheid</t>
+  </si>
+  <si>
+    <t>13. Testen op toegankelijkheid van de applicatie</t>
+  </si>
+  <si>
+    <t>14. Produceren van een "software bill of materials" (SBoM)</t>
+  </si>
+  <si>
+    <t>15. Opslaan van artifacten</t>
+  </si>
+  <si>
+    <t>16. Registratie van incidenten bij gebruik en beheer</t>
+  </si>
+  <si>
+    <t>17. Bij het uitvoeren van operationeel beheer; uitrollen van de software in de productieomgeving</t>
   </si>
   <si>
     <t>M08</t>
@@ -1752,7 +1725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2224,21 +2197,21 @@
       <c r="D55" s="5"/>
     </row>
     <row r="56" spans="1:4">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6" t="s">
+      <c r="A56" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="7"/>
+      <c r="B56" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="4"/>
       <c r="D56" s="5"/>
     </row>
     <row r="57" spans="1:4">
-      <c r="A57" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B57" s="3" t="s">
+      <c r="A57" s="6"/>
+      <c r="B57" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="4"/>
+      <c r="C57" s="7"/>
       <c r="D57" s="5"/>
     </row>
     <row r="58" spans="1:4">
@@ -2370,87 +2343,87 @@
       <c r="D73" s="5"/>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6" t="s">
+      <c r="A74" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C74" s="7"/>
+      <c r="B74" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C74" s="4"/>
       <c r="D74" s="5"/>
     </row>
     <row r="75" spans="1:4">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C75" s="7"/>
+      <c r="A75" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C75" s="4"/>
       <c r="D75" s="5"/>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C76" s="4"/>
-      <c r="D76" s="5"/>
+      <c r="A76" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C77" s="4"/>
       <c r="D77" s="5"/>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
-      <c r="D78" s="1"/>
+      <c r="A78" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C78" s="4"/>
+      <c r="D78" s="5"/>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C79" s="4"/>
       <c r="D79" s="5"/>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C80" s="4"/>
       <c r="D80" s="5"/>
     </row>
     <row r="81" spans="1:4">
-      <c r="A81" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C81" s="4"/>
+      <c r="A81" s="6"/>
+      <c r="B81" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C81" s="7"/>
       <c r="D81" s="5"/>
     </row>
     <row r="82" spans="1:4">
-      <c r="A82" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B82" s="3" t="s">
+      <c r="A82" s="6"/>
+      <c r="B82" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C82" s="4"/>
+      <c r="C82" s="7"/>
       <c r="D82" s="5"/>
     </row>
     <row r="83" spans="1:4">
@@ -2470,69 +2443,69 @@
       <c r="D84" s="5"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="6"/>
-      <c r="B85" s="6" t="s">
+      <c r="A85" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C85" s="7"/>
+      <c r="B85" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C85" s="4"/>
       <c r="D85" s="5"/>
     </row>
     <row r="86" spans="1:4">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C86" s="7"/>
+      <c r="A86" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C86" s="4"/>
       <c r="D86" s="5"/>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C87" s="4"/>
       <c r="D87" s="5"/>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C88" s="4"/>
       <c r="D88" s="5"/>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C89" s="4"/>
       <c r="D89" s="5"/>
     </row>
     <row r="90" spans="1:4">
-      <c r="A90" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C90" s="4"/>
+      <c r="A90" s="6"/>
+      <c r="B90" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C90" s="7"/>
       <c r="D90" s="5"/>
     </row>
     <row r="91" spans="1:4">
-      <c r="A91" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B91" s="3" t="s">
+      <c r="A91" s="6"/>
+      <c r="B91" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C91" s="4"/>
+      <c r="C91" s="7"/>
       <c r="D91" s="5"/>
     </row>
     <row r="92" spans="1:4">
@@ -2632,98 +2605,82 @@
       <c r="D103" s="5"/>
     </row>
     <row r="104" spans="1:4">
-      <c r="A104" s="6"/>
-      <c r="B104" s="6" t="s">
+      <c r="A104" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C104" s="7"/>
+      <c r="B104" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C104" s="4"/>
       <c r="D104" s="5"/>
     </row>
     <row r="105" spans="1:4">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C105" s="7"/>
-      <c r="D105" s="5"/>
+      <c r="A105" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B105" s="1"/>
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C106" s="4"/>
       <c r="D106" s="5"/>
     </row>
     <row r="107" spans="1:4">
-      <c r="A107" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
-      <c r="D107" s="1"/>
+      <c r="A107" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C107" s="4"/>
+      <c r="D107" s="5"/>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C108" s="4"/>
       <c r="D108" s="5"/>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C109" s="4"/>
       <c r="D109" s="5"/>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C110" s="4"/>
       <c r="D110" s="5"/>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C111" s="4"/>
       <c r="D111" s="5"/>
-    </row>
-    <row r="112" spans="1:4">
-      <c r="A112" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C112" s="4"/>
-      <c r="D112" s="5"/>
-    </row>
-    <row r="113" spans="1:4">
-      <c r="A113" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C113" s="4"/>
-      <c r="D113" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2816,7 +2773,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C105">
+  <conditionalFormatting sqref="C106">
     <cfRule type="cellIs" dxfId="0" priority="389" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2830,7 +2787,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C106">
+  <conditionalFormatting sqref="C107">
     <cfRule type="cellIs" dxfId="0" priority="393" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2914,34 +2871,6 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C112">
-    <cfRule type="cellIs" dxfId="0" priority="413" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="414" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="415" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="416" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C113">
-    <cfRule type="cellIs" dxfId="0" priority="417" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="418" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="419" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="420" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C12">
     <cfRule type="cellIs" dxfId="0" priority="21" operator="equal">
       <formula>"voldoet"</formula>
@@ -3852,7 +3781,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C76">
+  <conditionalFormatting sqref="C77">
     <cfRule type="cellIs" dxfId="0" priority="277" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3866,7 +3795,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C77">
+  <conditionalFormatting sqref="C78">
     <cfRule type="cellIs" dxfId="0" priority="281" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4202,7 +4131,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="105">
+  <dataValidations count="103">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4410,12 +4339,12 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C75">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C76">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C77">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C78">
+      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C79">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4494,12 +4423,12 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C104">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C105">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C106">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C107">
+      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C108">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4510,12 +4439,6 @@
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C111">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C112">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C113">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4537,7 +4460,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4545,10 +4468,10 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Hoofdmaatregelen niet scoren bij self-assessments.
Maak het scoren van hoofdmaatregelen onmogelijk bij maatregelen met submaatregelen.

Closes #952.
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -76,7 +76,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -204,7 +204,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -240,7 +240,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -295,7 +295,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -395,7 +395,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -463,7 +463,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -596,7 +596,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -732,7 +732,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Tip: bepaal eerst de status per submaatregel en daarna de status van de hoofdmaatregel.</t>
+          <t>Bepaal a.u.b. de status per submaatregel.</t>
         </r>
       </text>
     </comment>
@@ -886,10 +886,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
   <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 04-03-2025.</t>
-  </si>
-  <si>
-    <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Bij maatregelen met submaatregelen hoeft alleen de status van de submaatregelen te worden ingevuld.</t>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 21-03-2025.</t>
+  </si>
+  <si>
+    <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Vul bij maatregelen met submaatregelen alleen de status van de submaatregelen in.</t>
   </si>
   <si>
     <t>Bij maatregelen die primair door een project moeten worden toegepast geeft de status aan in hoevere het project dat doet. Bij maatregelen die primair door ICTU moeten worden toegepast geeft de status aan in hoeverre ICTU dat doet, gezien vanuit het perspectief van het project.</t>
@@ -1379,13 +1379,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFED32D"/>
+        <fgColor rgb="FFFFFFA5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFA5"/>
+        <fgColor rgb="FFFED32D"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1416,14 +1416,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" indent="1" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1822,40 +1822,40 @@
       <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="5"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="5"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
@@ -1864,160 +1864,160 @@
       <c r="B12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="5"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="5"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="4"/>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="5"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="4"/>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="5"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="5"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="4"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="5"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="4"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="5"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="4"/>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="5"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="5"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="5"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="5"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6" t="s">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="5"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6" t="s">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="5"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="4"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6" t="s">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="5"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="4"/>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6" t="s">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="5"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6" t="s">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="5"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6" t="s">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="5"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6" t="s">
+      <c r="A30" s="5"/>
+      <c r="B30" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="5"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6" t="s">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="5"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="3" t="s">
@@ -2026,32 +2026,32 @@
       <c r="B32" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="5"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6" t="s">
+      <c r="A33" s="5"/>
+      <c r="B33" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="5"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="4"/>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6" t="s">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="5"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="4"/>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6" t="s">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="5"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="3" t="s">
@@ -2060,56 +2060,56 @@
       <c r="B36" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="6"/>
-      <c r="B37" s="6" t="s">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="5"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="6"/>
-      <c r="B38" s="6" t="s">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="5"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="4"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="6"/>
-      <c r="B39" s="6" t="s">
+      <c r="A39" s="5"/>
+      <c r="B39" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="5"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="4"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="6"/>
-      <c r="B40" s="6" t="s">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="5"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="4"/>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="6"/>
-      <c r="B41" s="6" t="s">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C41" s="7"/>
-      <c r="D41" s="5"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="4"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6" t="s">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="5"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="4"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="3" t="s">
@@ -2118,8 +2118,8 @@
       <c r="B43" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="5"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="4"/>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="3" t="s">
@@ -2128,8 +2128,8 @@
       <c r="B44" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="5"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="4"/>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="3" t="s">
@@ -2138,8 +2138,8 @@
       <c r="B45" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="5"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="4"/>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="3" t="s">
@@ -2148,88 +2148,88 @@
       <c r="B46" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="5"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="4"/>
     </row>
     <row r="47" spans="1:4">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6" t="s">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C47" s="7"/>
-      <c r="D47" s="5"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="4"/>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="6"/>
-      <c r="B48" s="6" t="s">
+      <c r="A48" s="5"/>
+      <c r="B48" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="7"/>
-      <c r="D48" s="5"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="4"/>
     </row>
     <row r="49" spans="1:4">
-      <c r="A49" s="6"/>
-      <c r="B49" s="6" t="s">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C49" s="7"/>
-      <c r="D49" s="5"/>
+      <c r="C49" s="6"/>
+      <c r="D49" s="4"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6" t="s">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C50" s="7"/>
-      <c r="D50" s="5"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="4"/>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6" t="s">
+      <c r="A51" s="5"/>
+      <c r="B51" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C51" s="7"/>
-      <c r="D51" s="5"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="4"/>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6" t="s">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C52" s="7"/>
-      <c r="D52" s="5"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="4"/>
     </row>
     <row r="53" spans="1:4">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6" t="s">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C53" s="7"/>
-      <c r="D53" s="5"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="4"/>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6" t="s">
+      <c r="A54" s="5"/>
+      <c r="B54" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C54" s="7"/>
-      <c r="D54" s="5"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="4"/>
     </row>
     <row r="55" spans="1:4">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6" t="s">
+      <c r="A55" s="5"/>
+      <c r="B55" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C55" s="7"/>
-      <c r="D55" s="5"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="4"/>
     </row>
     <row r="56" spans="1:4">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6" t="s">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="7"/>
-      <c r="D56" s="5"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="4"/>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="3" t="s">
@@ -2238,152 +2238,152 @@
       <c r="B57" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="4"/>
-      <c r="D57" s="5"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="4"/>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6" t="s">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C58" s="7"/>
-      <c r="D58" s="5"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="4"/>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6" t="s">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C59" s="7"/>
-      <c r="D59" s="5"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="4"/>
     </row>
     <row r="60" spans="1:4">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6" t="s">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C60" s="7"/>
-      <c r="D60" s="5"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="4"/>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6" t="s">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="5"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="4"/>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6" t="s">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C62" s="7"/>
-      <c r="D62" s="5"/>
+      <c r="C62" s="6"/>
+      <c r="D62" s="4"/>
     </row>
     <row r="63" spans="1:4">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6" t="s">
+      <c r="A63" s="5"/>
+      <c r="B63" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C63" s="7"/>
-      <c r="D63" s="5"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="4"/>
     </row>
     <row r="64" spans="1:4">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6" t="s">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C64" s="7"/>
-      <c r="D64" s="5"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="4"/>
     </row>
     <row r="65" spans="1:4">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6" t="s">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C65" s="7"/>
-      <c r="D65" s="5"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="4"/>
     </row>
     <row r="66" spans="1:4">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6" t="s">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C66" s="7"/>
-      <c r="D66" s="5"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="4"/>
     </row>
     <row r="67" spans="1:4">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6" t="s">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C67" s="7"/>
-      <c r="D67" s="5"/>
+      <c r="C67" s="6"/>
+      <c r="D67" s="4"/>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6" t="s">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C68" s="7"/>
-      <c r="D68" s="5"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="4"/>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6" t="s">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C69" s="7"/>
-      <c r="D69" s="5"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="4"/>
     </row>
     <row r="70" spans="1:4">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6" t="s">
+      <c r="A70" s="5"/>
+      <c r="B70" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C70" s="7"/>
-      <c r="D70" s="5"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="4"/>
     </row>
     <row r="71" spans="1:4">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6" t="s">
+      <c r="A71" s="5"/>
+      <c r="B71" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C71" s="7"/>
-      <c r="D71" s="5"/>
+      <c r="C71" s="6"/>
+      <c r="D71" s="4"/>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6" t="s">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C72" s="7"/>
-      <c r="D72" s="5"/>
+      <c r="C72" s="6"/>
+      <c r="D72" s="4"/>
     </row>
     <row r="73" spans="1:4">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6" t="s">
+      <c r="A73" s="5"/>
+      <c r="B73" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C73" s="7"/>
-      <c r="D73" s="5"/>
+      <c r="C73" s="6"/>
+      <c r="D73" s="4"/>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6" t="s">
+      <c r="A74" s="5"/>
+      <c r="B74" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C74" s="7"/>
-      <c r="D74" s="5"/>
+      <c r="C74" s="6"/>
+      <c r="D74" s="4"/>
     </row>
     <row r="75" spans="1:4">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6" t="s">
+      <c r="A75" s="5"/>
+      <c r="B75" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C75" s="7"/>
-      <c r="D75" s="5"/>
+      <c r="C75" s="6"/>
+      <c r="D75" s="4"/>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="3" t="s">
@@ -2392,8 +2392,8 @@
       <c r="B76" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C76" s="4"/>
-      <c r="D76" s="5"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="4"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="3" t="s">
@@ -2402,8 +2402,8 @@
       <c r="B77" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C77" s="4"/>
-      <c r="D77" s="5"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="4"/>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="1" t="s">
@@ -2420,8 +2420,8 @@
       <c r="B79" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C79" s="4"/>
-      <c r="D79" s="5"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="4"/>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="3" t="s">
@@ -2430,8 +2430,8 @@
       <c r="B80" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C80" s="4"/>
-      <c r="D80" s="5"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="4"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="3" t="s">
@@ -2440,8 +2440,8 @@
       <c r="B81" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C81" s="4"/>
-      <c r="D81" s="5"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="4"/>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="3" t="s">
@@ -2450,40 +2450,40 @@
       <c r="B82" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C82" s="4"/>
-      <c r="D82" s="5"/>
+      <c r="C82" s="3"/>
+      <c r="D82" s="4"/>
     </row>
     <row r="83" spans="1:4">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6" t="s">
+      <c r="A83" s="5"/>
+      <c r="B83" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C83" s="7"/>
-      <c r="D83" s="5"/>
+      <c r="C83" s="6"/>
+      <c r="D83" s="4"/>
     </row>
     <row r="84" spans="1:4">
-      <c r="A84" s="6"/>
-      <c r="B84" s="6" t="s">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C84" s="7"/>
-      <c r="D84" s="5"/>
+      <c r="C84" s="6"/>
+      <c r="D84" s="4"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="6"/>
-      <c r="B85" s="6" t="s">
+      <c r="A85" s="5"/>
+      <c r="B85" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C85" s="7"/>
-      <c r="D85" s="5"/>
+      <c r="C85" s="6"/>
+      <c r="D85" s="4"/>
     </row>
     <row r="86" spans="1:4">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6" t="s">
+      <c r="A86" s="5"/>
+      <c r="B86" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C86" s="7"/>
-      <c r="D86" s="5"/>
+      <c r="C86" s="6"/>
+      <c r="D86" s="4"/>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="3" t="s">
@@ -2492,8 +2492,8 @@
       <c r="B87" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C87" s="4"/>
-      <c r="D87" s="5"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="4"/>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="3" t="s">
@@ -2502,8 +2502,8 @@
       <c r="B88" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C88" s="4"/>
-      <c r="D88" s="5"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="4"/>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="3" t="s">
@@ -2512,8 +2512,8 @@
       <c r="B89" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C89" s="4"/>
-      <c r="D89" s="5"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="4"/>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="3" t="s">
@@ -2522,8 +2522,8 @@
       <c r="B90" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C90" s="4"/>
-      <c r="D90" s="5"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="4"/>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="3" t="s">
@@ -2532,120 +2532,120 @@
       <c r="B91" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C91" s="4"/>
-      <c r="D91" s="5"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="4"/>
     </row>
     <row r="92" spans="1:4">
-      <c r="A92" s="6"/>
-      <c r="B92" s="6" t="s">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C92" s="7"/>
-      <c r="D92" s="5"/>
+      <c r="C92" s="6"/>
+      <c r="D92" s="4"/>
     </row>
     <row r="93" spans="1:4">
-      <c r="A93" s="6"/>
-      <c r="B93" s="6" t="s">
+      <c r="A93" s="5"/>
+      <c r="B93" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C93" s="7"/>
-      <c r="D93" s="5"/>
+      <c r="C93" s="6"/>
+      <c r="D93" s="4"/>
     </row>
     <row r="94" spans="1:4">
-      <c r="A94" s="6"/>
-      <c r="B94" s="6" t="s">
+      <c r="A94" s="5"/>
+      <c r="B94" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C94" s="7"/>
-      <c r="D94" s="5"/>
+      <c r="C94" s="6"/>
+      <c r="D94" s="4"/>
     </row>
     <row r="95" spans="1:4">
-      <c r="A95" s="6"/>
-      <c r="B95" s="6" t="s">
+      <c r="A95" s="5"/>
+      <c r="B95" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C95" s="7"/>
-      <c r="D95" s="5"/>
+      <c r="C95" s="6"/>
+      <c r="D95" s="4"/>
     </row>
     <row r="96" spans="1:4">
-      <c r="A96" s="6"/>
-      <c r="B96" s="6" t="s">
+      <c r="A96" s="5"/>
+      <c r="B96" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C96" s="7"/>
-      <c r="D96" s="5"/>
+      <c r="C96" s="6"/>
+      <c r="D96" s="4"/>
     </row>
     <row r="97" spans="1:4">
-      <c r="A97" s="6"/>
-      <c r="B97" s="6" t="s">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C97" s="7"/>
-      <c r="D97" s="5"/>
+      <c r="C97" s="6"/>
+      <c r="D97" s="4"/>
     </row>
     <row r="98" spans="1:4">
-      <c r="A98" s="6"/>
-      <c r="B98" s="6" t="s">
+      <c r="A98" s="5"/>
+      <c r="B98" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C98" s="7"/>
-      <c r="D98" s="5"/>
+      <c r="C98" s="6"/>
+      <c r="D98" s="4"/>
     </row>
     <row r="99" spans="1:4">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6" t="s">
+      <c r="A99" s="5"/>
+      <c r="B99" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C99" s="7"/>
-      <c r="D99" s="5"/>
+      <c r="C99" s="6"/>
+      <c r="D99" s="4"/>
     </row>
     <row r="100" spans="1:4">
-      <c r="A100" s="6"/>
-      <c r="B100" s="6" t="s">
+      <c r="A100" s="5"/>
+      <c r="B100" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C100" s="7"/>
-      <c r="D100" s="5"/>
+      <c r="C100" s="6"/>
+      <c r="D100" s="4"/>
     </row>
     <row r="101" spans="1:4">
-      <c r="A101" s="6"/>
-      <c r="B101" s="6" t="s">
+      <c r="A101" s="5"/>
+      <c r="B101" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C101" s="7"/>
-      <c r="D101" s="5"/>
+      <c r="C101" s="6"/>
+      <c r="D101" s="4"/>
     </row>
     <row r="102" spans="1:4">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6" t="s">
+      <c r="A102" s="5"/>
+      <c r="B102" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C102" s="7"/>
-      <c r="D102" s="5"/>
+      <c r="C102" s="6"/>
+      <c r="D102" s="4"/>
     </row>
     <row r="103" spans="1:4">
-      <c r="A103" s="6"/>
-      <c r="B103" s="6" t="s">
+      <c r="A103" s="5"/>
+      <c r="B103" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="C103" s="7"/>
-      <c r="D103" s="5"/>
+      <c r="C103" s="6"/>
+      <c r="D103" s="4"/>
     </row>
     <row r="104" spans="1:4">
-      <c r="A104" s="6"/>
-      <c r="B104" s="6" t="s">
+      <c r="A104" s="5"/>
+      <c r="B104" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C104" s="7"/>
-      <c r="D104" s="5"/>
+      <c r="C104" s="6"/>
+      <c r="D104" s="4"/>
     </row>
     <row r="105" spans="1:4">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6" t="s">
+      <c r="A105" s="5"/>
+      <c r="B105" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C105" s="7"/>
-      <c r="D105" s="5"/>
+      <c r="C105" s="6"/>
+      <c r="D105" s="4"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="3" t="s">
@@ -2654,8 +2654,8 @@
       <c r="B106" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C106" s="4"/>
-      <c r="D106" s="5"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="4"/>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="1" t="s">
@@ -2672,8 +2672,8 @@
       <c r="B108" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C108" s="4"/>
-      <c r="D108" s="5"/>
+      <c r="C108" s="7"/>
+      <c r="D108" s="4"/>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="3" t="s">
@@ -2682,8 +2682,8 @@
       <c r="B109" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C109" s="4"/>
-      <c r="D109" s="5"/>
+      <c r="C109" s="7"/>
+      <c r="D109" s="4"/>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="3" t="s">
@@ -2692,8 +2692,8 @@
       <c r="B110" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C110" s="4"/>
-      <c r="D110" s="5"/>
+      <c r="C110" s="7"/>
+      <c r="D110" s="4"/>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="3" t="s">
@@ -2702,8 +2702,8 @@
       <c r="B111" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C111" s="4"/>
-      <c r="D111" s="5"/>
+      <c r="C111" s="7"/>
+      <c r="D111" s="4"/>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="3" t="s">
@@ -2712,8 +2712,8 @@
       <c r="B112" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C112" s="4"/>
-      <c r="D112" s="5"/>
+      <c r="C112" s="7"/>
+      <c r="D112" s="4"/>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="3" t="s">
@@ -2722,8 +2722,8 @@
       <c r="B113" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C113" s="4"/>
-      <c r="D113" s="5"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2733,6 +2733,146 @@
     <mergeCell ref="A4:D4"/>
   </mergeCells>
   <conditionalFormatting sqref="C10">
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="11" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="12" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C100">
+    <cfRule type="cellIs" dxfId="0" priority="337" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="338" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="339" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="340" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C101">
+    <cfRule type="cellIs" dxfId="0" priority="341" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="342" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="343" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="344" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C102">
+    <cfRule type="cellIs" dxfId="0" priority="345" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="346" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="347" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="348" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C103">
+    <cfRule type="cellIs" dxfId="0" priority="349" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="350" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="351" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="352" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C104">
+    <cfRule type="cellIs" dxfId="0" priority="353" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="354" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="355" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="356" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C105">
+    <cfRule type="cellIs" dxfId="0" priority="357" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="358" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="359" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="360" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C106">
+    <cfRule type="cellIs" dxfId="0" priority="361" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="362" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="363" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="364" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C108">
+    <cfRule type="cellIs" dxfId="0" priority="365" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="366" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="367" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="368" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C109">
+    <cfRule type="cellIs" dxfId="0" priority="369" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="370" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="371" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="372" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
     <cfRule type="cellIs" dxfId="0" priority="13" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2746,21 +2886,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C100">
-    <cfRule type="cellIs" dxfId="0" priority="369" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="370" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="371" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="372" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C101">
+  <conditionalFormatting sqref="C110">
     <cfRule type="cellIs" dxfId="0" priority="373" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2774,7 +2900,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C102">
+  <conditionalFormatting sqref="C111">
     <cfRule type="cellIs" dxfId="0" priority="377" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2788,7 +2914,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C103">
+  <conditionalFormatting sqref="C112">
     <cfRule type="cellIs" dxfId="0" priority="381" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2802,7 +2928,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C104">
+  <conditionalFormatting sqref="C113">
     <cfRule type="cellIs" dxfId="0" priority="385" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2816,63 +2942,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C105">
-    <cfRule type="cellIs" dxfId="0" priority="389" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="390" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="391" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="392" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C106">
-    <cfRule type="cellIs" dxfId="0" priority="393" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="394" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="395" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="396" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C108">
-    <cfRule type="cellIs" dxfId="0" priority="397" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="398" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="399" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="400" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C109">
-    <cfRule type="cellIs" dxfId="0" priority="401" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="402" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="403" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="404" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
+  <conditionalFormatting sqref="C13">
     <cfRule type="cellIs" dxfId="0" priority="17" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2886,63 +2956,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C110">
-    <cfRule type="cellIs" dxfId="0" priority="405" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="406" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="407" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="408" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C111">
-    <cfRule type="cellIs" dxfId="0" priority="409" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="410" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="411" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="412" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C112">
-    <cfRule type="cellIs" dxfId="0" priority="413" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="414" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="415" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="416" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C113">
-    <cfRule type="cellIs" dxfId="0" priority="417" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="418" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="419" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="420" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C12">
+  <conditionalFormatting sqref="C14">
     <cfRule type="cellIs" dxfId="0" priority="21" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2956,7 +2970,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
+  <conditionalFormatting sqref="C15">
     <cfRule type="cellIs" dxfId="0" priority="25" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2970,7 +2984,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C14">
+  <conditionalFormatting sqref="C16">
     <cfRule type="cellIs" dxfId="0" priority="29" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2984,7 +2998,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C15">
+  <conditionalFormatting sqref="C17">
     <cfRule type="cellIs" dxfId="0" priority="33" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -2998,7 +3012,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
+  <conditionalFormatting sqref="C18">
     <cfRule type="cellIs" dxfId="0" priority="37" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3012,7 +3026,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
+  <conditionalFormatting sqref="C19">
     <cfRule type="cellIs" dxfId="0" priority="41" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3026,7 +3040,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
+  <conditionalFormatting sqref="C20">
     <cfRule type="cellIs" dxfId="0" priority="45" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3040,7 +3054,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
+  <conditionalFormatting sqref="C21">
     <cfRule type="cellIs" dxfId="0" priority="49" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3054,7 +3068,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
+  <conditionalFormatting sqref="C22">
     <cfRule type="cellIs" dxfId="0" priority="53" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3068,7 +3082,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
+  <conditionalFormatting sqref="C23">
     <cfRule type="cellIs" dxfId="0" priority="57" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3082,7 +3096,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
+  <conditionalFormatting sqref="C24">
     <cfRule type="cellIs" dxfId="0" priority="61" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3096,7 +3110,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
+  <conditionalFormatting sqref="C25">
     <cfRule type="cellIs" dxfId="0" priority="65" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3110,7 +3124,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
+  <conditionalFormatting sqref="C26">
     <cfRule type="cellIs" dxfId="0" priority="69" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3124,7 +3138,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
+  <conditionalFormatting sqref="C27">
     <cfRule type="cellIs" dxfId="0" priority="73" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3138,7 +3152,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C26">
+  <conditionalFormatting sqref="C28">
     <cfRule type="cellIs" dxfId="0" priority="77" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3152,7 +3166,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27">
+  <conditionalFormatting sqref="C29">
     <cfRule type="cellIs" dxfId="0" priority="81" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3166,7 +3180,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28">
+  <conditionalFormatting sqref="C30">
     <cfRule type="cellIs" dxfId="0" priority="85" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3180,7 +3194,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29">
+  <conditionalFormatting sqref="C31">
     <cfRule type="cellIs" dxfId="0" priority="89" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3194,7 +3208,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C30">
+  <conditionalFormatting sqref="C33">
     <cfRule type="cellIs" dxfId="0" priority="93" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3208,7 +3222,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
+  <conditionalFormatting sqref="C34">
     <cfRule type="cellIs" dxfId="0" priority="97" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3222,7 +3236,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C32">
+  <conditionalFormatting sqref="C35">
     <cfRule type="cellIs" dxfId="0" priority="101" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3236,7 +3250,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33">
+  <conditionalFormatting sqref="C37">
     <cfRule type="cellIs" dxfId="0" priority="105" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3250,7 +3264,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C34">
+  <conditionalFormatting sqref="C38">
     <cfRule type="cellIs" dxfId="0" priority="109" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3264,7 +3278,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C35">
+  <conditionalFormatting sqref="C39">
     <cfRule type="cellIs" dxfId="0" priority="113" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3278,7 +3292,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C36">
+  <conditionalFormatting sqref="C40">
     <cfRule type="cellIs" dxfId="0" priority="117" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3292,7 +3306,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37">
+  <conditionalFormatting sqref="C41">
     <cfRule type="cellIs" dxfId="0" priority="121" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3306,7 +3320,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C38">
+  <conditionalFormatting sqref="C42">
     <cfRule type="cellIs" dxfId="0" priority="125" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3320,7 +3334,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C39">
+  <conditionalFormatting sqref="C43">
     <cfRule type="cellIs" dxfId="0" priority="129" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3334,7 +3348,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C40">
+  <conditionalFormatting sqref="C44">
     <cfRule type="cellIs" dxfId="0" priority="133" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3348,7 +3362,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C41">
+  <conditionalFormatting sqref="C45">
     <cfRule type="cellIs" dxfId="0" priority="137" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3362,7 +3376,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C42">
+  <conditionalFormatting sqref="C47">
     <cfRule type="cellIs" dxfId="0" priority="141" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3376,7 +3390,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C43">
+  <conditionalFormatting sqref="C48">
     <cfRule type="cellIs" dxfId="0" priority="145" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3390,7 +3404,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C44">
+  <conditionalFormatting sqref="C49">
     <cfRule type="cellIs" dxfId="0" priority="149" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3404,7 +3418,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C45">
+  <conditionalFormatting sqref="C50">
     <cfRule type="cellIs" dxfId="0" priority="153" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3418,7 +3432,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46">
+  <conditionalFormatting sqref="C51">
     <cfRule type="cellIs" dxfId="0" priority="157" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3432,7 +3446,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C47">
+  <conditionalFormatting sqref="C52">
     <cfRule type="cellIs" dxfId="0" priority="161" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3446,7 +3460,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48">
+  <conditionalFormatting sqref="C53">
     <cfRule type="cellIs" dxfId="0" priority="165" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3460,7 +3474,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C49">
+  <conditionalFormatting sqref="C54">
     <cfRule type="cellIs" dxfId="0" priority="169" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3474,7 +3488,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C50">
+  <conditionalFormatting sqref="C55">
     <cfRule type="cellIs" dxfId="0" priority="173" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3488,7 +3502,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C51">
+  <conditionalFormatting sqref="C56">
     <cfRule type="cellIs" dxfId="0" priority="177" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3502,7 +3516,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C52">
+  <conditionalFormatting sqref="C58">
     <cfRule type="cellIs" dxfId="0" priority="181" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3516,7 +3530,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C53">
+  <conditionalFormatting sqref="C59">
     <cfRule type="cellIs" dxfId="0" priority="185" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3530,7 +3544,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C54">
+  <conditionalFormatting sqref="C60">
     <cfRule type="cellIs" dxfId="0" priority="189" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3544,7 +3558,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C55">
+  <conditionalFormatting sqref="C61">
     <cfRule type="cellIs" dxfId="0" priority="193" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3558,7 +3572,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C56">
+  <conditionalFormatting sqref="C62">
     <cfRule type="cellIs" dxfId="0" priority="197" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3572,7 +3586,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C57">
+  <conditionalFormatting sqref="C63">
     <cfRule type="cellIs" dxfId="0" priority="201" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3586,7 +3600,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C58">
+  <conditionalFormatting sqref="C64">
     <cfRule type="cellIs" dxfId="0" priority="205" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3600,7 +3614,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C59">
+  <conditionalFormatting sqref="C65">
     <cfRule type="cellIs" dxfId="0" priority="209" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3614,7 +3628,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C60">
+  <conditionalFormatting sqref="C66">
     <cfRule type="cellIs" dxfId="0" priority="213" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3628,7 +3642,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C61">
+  <conditionalFormatting sqref="C67">
     <cfRule type="cellIs" dxfId="0" priority="217" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3642,7 +3656,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C62">
+  <conditionalFormatting sqref="C68">
     <cfRule type="cellIs" dxfId="0" priority="221" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3656,7 +3670,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C63">
+  <conditionalFormatting sqref="C69">
     <cfRule type="cellIs" dxfId="0" priority="225" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3670,7 +3684,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C64">
+  <conditionalFormatting sqref="C70">
     <cfRule type="cellIs" dxfId="0" priority="229" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3684,7 +3698,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C65">
+  <conditionalFormatting sqref="C71">
     <cfRule type="cellIs" dxfId="0" priority="233" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3698,7 +3712,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C66">
+  <conditionalFormatting sqref="C72">
     <cfRule type="cellIs" dxfId="0" priority="237" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3712,7 +3726,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C67">
+  <conditionalFormatting sqref="C73">
     <cfRule type="cellIs" dxfId="0" priority="241" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3726,7 +3740,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C68">
+  <conditionalFormatting sqref="C74">
     <cfRule type="cellIs" dxfId="0" priority="245" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3740,7 +3754,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C69">
+  <conditionalFormatting sqref="C75">
     <cfRule type="cellIs" dxfId="0" priority="249" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3754,7 +3768,49 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
+  <conditionalFormatting sqref="C76">
+    <cfRule type="cellIs" dxfId="0" priority="253" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="254" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="255" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="256" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C77">
+    <cfRule type="cellIs" dxfId="0" priority="257" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="258" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="259" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="260" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C79">
+    <cfRule type="cellIs" dxfId="0" priority="261" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="262" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="263" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="264" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3768,49 +3824,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C70">
-    <cfRule type="cellIs" dxfId="0" priority="253" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="254" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="255" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="256" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C71">
-    <cfRule type="cellIs" dxfId="0" priority="257" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="258" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="259" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="260" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C72">
-    <cfRule type="cellIs" dxfId="0" priority="261" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="262" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="263" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="264" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C73">
+  <conditionalFormatting sqref="C80">
     <cfRule type="cellIs" dxfId="0" priority="265" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3824,7 +3838,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C74">
+  <conditionalFormatting sqref="C81">
     <cfRule type="cellIs" dxfId="0" priority="269" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3838,7 +3852,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C75">
+  <conditionalFormatting sqref="C83">
     <cfRule type="cellIs" dxfId="0" priority="273" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3852,7 +3866,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C76">
+  <conditionalFormatting sqref="C84">
     <cfRule type="cellIs" dxfId="0" priority="277" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3866,7 +3880,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C77">
+  <conditionalFormatting sqref="C85">
     <cfRule type="cellIs" dxfId="0" priority="281" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3880,7 +3894,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C79">
+  <conditionalFormatting sqref="C86">
     <cfRule type="cellIs" dxfId="0" priority="285" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3894,7 +3908,49 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
+  <conditionalFormatting sqref="C87">
+    <cfRule type="cellIs" dxfId="0" priority="289" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="290" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="291" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="292" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C88">
+    <cfRule type="cellIs" dxfId="0" priority="293" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="294" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="295" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="296" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C89">
+    <cfRule type="cellIs" dxfId="0" priority="297" operator="equal">
+      <formula>"voldoet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="298" operator="equal">
+      <formula>"voldoet deels"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="299" operator="equal">
+      <formula>"voldoet niet"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="300" operator="equal">
+      <formula>"niet van toepassing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
     <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3908,49 +3964,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C80">
-    <cfRule type="cellIs" dxfId="0" priority="289" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="290" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="291" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="292" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C81">
-    <cfRule type="cellIs" dxfId="0" priority="293" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="294" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="295" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="296" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C82">
-    <cfRule type="cellIs" dxfId="0" priority="297" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="298" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="299" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="300" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C83">
+  <conditionalFormatting sqref="C90">
     <cfRule type="cellIs" dxfId="0" priority="301" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3964,7 +3978,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C84">
+  <conditionalFormatting sqref="C92">
     <cfRule type="cellIs" dxfId="0" priority="305" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3978,7 +3992,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C85">
+  <conditionalFormatting sqref="C93">
     <cfRule type="cellIs" dxfId="0" priority="309" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -3992,7 +4006,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C86">
+  <conditionalFormatting sqref="C94">
     <cfRule type="cellIs" dxfId="0" priority="313" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4006,7 +4020,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C87">
+  <conditionalFormatting sqref="C95">
     <cfRule type="cellIs" dxfId="0" priority="317" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4020,7 +4034,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C88">
+  <conditionalFormatting sqref="C96">
     <cfRule type="cellIs" dxfId="0" priority="321" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4034,7 +4048,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C89">
+  <conditionalFormatting sqref="C97">
     <cfRule type="cellIs" dxfId="0" priority="325" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4048,21 +4062,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="11" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="12" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C90">
+  <conditionalFormatting sqref="C98">
     <cfRule type="cellIs" dxfId="0" priority="329" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4076,7 +4076,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C91">
+  <conditionalFormatting sqref="C99">
     <cfRule type="cellIs" dxfId="0" priority="333" operator="equal">
       <formula>"voldoet"</formula>
     </cfRule>
@@ -4090,122 +4090,7 @@
       <formula>"niet van toepassing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C92">
-    <cfRule type="cellIs" dxfId="0" priority="337" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="338" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="339" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="340" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C93">
-    <cfRule type="cellIs" dxfId="0" priority="341" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="342" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="343" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="344" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C94">
-    <cfRule type="cellIs" dxfId="0" priority="345" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="346" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="347" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="348" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C95">
-    <cfRule type="cellIs" dxfId="0" priority="349" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="350" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="351" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="352" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C96">
-    <cfRule type="cellIs" dxfId="0" priority="353" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="354" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="355" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="356" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C97">
-    <cfRule type="cellIs" dxfId="0" priority="357" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="358" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="359" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="360" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C98">
-    <cfRule type="cellIs" dxfId="0" priority="361" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="362" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="363" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="364" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C99">
-    <cfRule type="cellIs" dxfId="0" priority="365" operator="equal">
-      <formula>"voldoet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="366" operator="equal">
-      <formula>"voldoet deels"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="367" operator="equal">
-      <formula>"voldoet niet"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="368" operator="equal">
-      <formula>"niet van toepassing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="105">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
+  <dataValidations count="97">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4218,9 +4103,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C11">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C12">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C13">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4278,9 +4160,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C31">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C32">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C33">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4290,9 +4169,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C35">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C36">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C37">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4320,9 +4196,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C45">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C46">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C47">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4353,9 +4226,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C56">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C57">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C58">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4425,9 +4295,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C81">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C82">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C83">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
@@ -4450,9 +4317,6 @@
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C90">
-      <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C91">
       <formula1>"voldoet,voldoet deels,voldoet niet,niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C92">

</xml_diff>

<commit_message>
Mark measure and submeasure titles in the XML
</commit_message>
<xml_diff>
--- a/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
+++ b/docs/wip/ICTU-Kwaliteitsaanpak-Checklist.xlsx
@@ -62,6 +62,7 @@
 Als een DPIA niet nodig is, dan is een verklaring daaromtrent vereist.
 Impact assessment mensenrechten en algoritmes
 Een impact assessment voor mensenrechten bij de inzet van algoritmes is een instrument voor discussie en besluitvorming door overheidsorganen over de ontwikkeling en/of inzet van een algoritmisch systeem. Met een dergelijke impact assessment kan een interdisciplinaire dialoog gevoerd worden tussen relevante partijen bij de afweging om wel of niet een algoritmische toepassing te gaan ontwikkelen. En het helpt om de gekozen ontwikkeling en implementatie vervolgens op een verantwoorde manier te doen. In het IAMA worden verbanden gelegd met relevante regels, instrumenten en toetskaders op het gebied van algoritmen.
+Een IAMA wordt ingezet in alle gevallen waarin een overheidsorgaan overweegt een algoritme te (laten) ontwikkelen, in te kopen, aan te passen en/of in te gaan zetten.
 Zie https://www.rijksoverheid.nl/documenten/rapporten/2021/02/25/impact-assessment-mensenrechten-en-algoritmes.
 Voor meer informatie over het gezamenlijk gebruik van IAMA en DPIA, zie https://www.cip-overheid.nl/media/av0dmahv/20230614-gezamenlijk-gebruik-iama-en-model-dpia-rijksdienst-v1-0.pdf.
 Projectstartarchitectuur en solution architectuur
@@ -487,9 +488,9 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">M23: Het project zorgt voor de aanwezigheid van kennis van en ervaring met de Kwaliteitsaanpak
-De software delivery manager zorgt ervoor dat bij nieuwe projecten wordt gestart met ten minste twee projectleden die bekend zijn met de Kwaliteitsaanpak. Projectleden die nog niet bekend zijn met de Kwaliteitsaanpak krijgen uitleg over de inhoud en achtergrond van de Kwaliteitsaanpak.
+De software delivery manager zorgt ervoor dat bij nieuwe projecten wordt gestart met ten minste twee projectleden die bekend zijn met de Kwaliteitsaanpak. Projectleden, inclusief projectleider, die nog niet bekend zijn met de Kwaliteitsaanpak krijgen uitleg over de inhoud en achtergrond van de Kwaliteitsaanpak.
 Rationale
-Het inzetten van teamleden die bekend zijn met de Kwaliteitsaanpak zorgt voor een soepeler start van een nieuw project omdat zij bekend zijn met de inhoud van de Kwaliteitsaanpak, zoals kwaliteitsnormen en tools, en omdat zij al doende nieuwe teamleden bekend kunnen maken met de Kwaliteitsaanpak.
+Het inzetten van projectleden die bekend zijn met de Kwaliteitsaanpak zorgt voor een soepeler start van een nieuw project omdat zij bekend zijn met de inhoud van de Kwaliteitsaanpak, zoals kwaliteitsnormen en tools, en omdat zij al doende nieuwe projectleden bekend kunnen maken met de Kwaliteitsaanpak.
 </t>
         </r>
       </text>
@@ -816,7 +817,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="138">
   <si>
-    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 11-04-2025.</t>
+    <t>Onderstaande checklist kan gebruikt worden voor het uitvoeren van een assessment tegen de ICTU Kwaliteitsaanpak Softwareontwikkeling versie wip, 19-09-2025.</t>
   </si>
   <si>
     <t>Gebruik de 'Status' kolom om aan te geven in hoeverre een maatregel uit de Kwaliteitsaanpak is toegepast. Vul bij maatregelen met submaatregelen alleen de status van de submaatregelen in.</t>

</xml_diff>